<commit_message>
updating project diary and group discussion
</commit_message>
<xml_diff>
--- a/Project Plan.xlsx
+++ b/Project Plan.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Semester 2\ETC5521\Project 1\project-part-1-p1-wallaby\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{677154CC-2F96-466D-9842-6066FDA5573E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F590E7D2-60E1-4B99-8A20-BF4FE8E552E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{08FA5D9B-BDCD-4B0C-BBC1-0603E7BA2D97}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{08FA5D9B-BDCD-4B0C-BBC1-0603E7BA2D97}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Plan" sheetId="1" r:id="rId1"/>
+    <sheet name="Team Analysis" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="94">
   <si>
     <t>Section</t>
   </si>
@@ -121,13 +122,665 @@
   </si>
   <si>
     <t>Create the concise conclusion</t>
+  </si>
+  <si>
+    <t>sub-question</t>
+  </si>
+  <si>
+    <t>How did leverage (debt-to-assets) and liquidity (current ratio) evolve during 2020–2022?</t>
+  </si>
+  <si>
+    <t>Did firm size influence financial resilience during the pandemic period?</t>
+  </si>
+  <si>
+    <t>How did profitability change across industries (2020–2022)?</t>
+  </si>
+  <si>
+    <t>variables</t>
+  </si>
+  <si>
+    <t>industry_group, year, ebit_margin_pct, ebitda_margin_pct, roa_pct, total_revenue_eur</t>
+  </si>
+  <si>
+    <t>total_liab_debt_eur     = `total_liabilities_and_debt_data14022`,</t>
+  </si>
+  <si>
+    <t>total_revenues_eur      = `total_revenues_data13004`,</t>
+  </si>
+  <si>
+    <t>solvency_ratio_pct      = `solvency_ratio_data31310`</t>
+  </si>
+  <si>
+    <t>company_name  = `company_name_name`,</t>
+  </si>
+  <si>
+    <t>company_id = nameid,</t>
+  </si>
+  <si>
+    <t>country    = `country_country`,</t>
+  </si>
+  <si>
+    <t>roa_pct    = `return_on_total_assets_data31015`,</t>
+  </si>
+  <si>
+    <t>gearing_pct= `gearing_data31315`,</t>
+  </si>
+  <si>
+    <t>nace_core_code   = `nace_rev_1_core_code_cnacecd`,</t>
+  </si>
+  <si>
+    <t>sic_core_code    = `us_sic_core_code_csicuscde`,</t>
+  </si>
+  <si>
+    <t>naics_core_code  = `naics_core_code_caics12cod`,</t>
+  </si>
+  <si>
+    <t>total_assets_eur = `total_assets_data13077`,</t>
+  </si>
+  <si>
+    <t>total_equity_eur = `total_shareholders_equity_data14041`,</t>
+  </si>
+  <si>
+    <t>net_sales_eur    = `net_sales_data13002`,</t>
+  </si>
+  <si>
+    <t>gross_sales_eur  = `gross_sales_data13000`,</t>
+  </si>
+  <si>
+    <t>ebit_margin_pct  = `ebit_margin_data31055`,</t>
+  </si>
+  <si>
+    <t>ebitda_margin_pct= `ebitda_margin_data31060`,</t>
+  </si>
+  <si>
+    <t>year = year,</t>
+  </si>
+  <si>
+    <t>1. Line trends of average EBIT margin by industry
+2. Boxplots of profitability (EBITDA margin) by industry and year
+3. Heatmap of change in ROA (2022 – 2020) by industry</t>
+  </si>
+  <si>
+    <t>debt_to_assets (derived), equity_ratio (derived),
+gearing_pct, solvency_ratio_pct,
+year, optional industry_group</t>
+  </si>
+  <si>
+    <t>size_group (derived from assets), year. Profitability: ebit_margin_pct and/or roa_pct. Stability: optional IQR or SD of profitability by size</t>
+  </si>
+  <si>
+    <t>Why this is relevant:</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Profitability (EBIT, EBITDA, ROA) directly reflects the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>operational and market impact</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> of the pandemic.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Industry breakdowns capture the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>uneven shock</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: travel and manufacturing shrank, while healthcare and ICT improved.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">This question links the macro shock (pandemic) to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>micro outcomes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (profit margins).</t>
+    </r>
+  </si>
+  <si>
+    <t>Why this is excellent:</t>
+  </si>
+  <si>
+    <t>It ties directly to “corporate financials” via performance metrics.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">It provides </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>comparative insight</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (sectoral resilience).</t>
+    </r>
+  </si>
+  <si>
+    <t>It is measurable using existing variables:</t>
+  </si>
+  <si>
+    <r>
+      <t>ebit_margin_pct</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>ebitda_margin_pct</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>roa_pct</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>industry_group</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Example visuals (you already planned):</t>
+  </si>
+  <si>
+    <t>1. Industry line trend (mean EBIT margin).</t>
+  </si>
+  <si>
+    <t>2. Boxplots of EBITDA margin by year.</t>
+  </si>
+  <si>
+    <t>3. ROA heatmap (change 2020→2022).</t>
+  </si>
+  <si>
+    <t>Q1</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The pandemic forced firms to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>restructure debt</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, affecting solvency and liquidity.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Leverage and solvency show </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>financial vulnerability</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>post-shock recovery</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> capacity.</t>
+    </r>
+  </si>
+  <si>
+    <t>Your dataset includes strong ratio variables for this:</t>
+  </si>
+  <si>
+    <r>
+      <t>gearing_pct</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>solvency_ratio_pct</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, and derived </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>debt_to_assets</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>equity_ratio</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">It examines </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>balance-sheet health</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, another pillar of corporate financials.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">It complements profitability (Q1) by exploring </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>risk exposure</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>It connects to corporate policy responses — e.g., borrowing in 2020, deleveraging later.</t>
+  </si>
+  <si>
+    <t>Example visuals:</t>
+  </si>
+  <si>
+    <t>1. Multi-indicator line trends (mean leverage/solvency).</t>
+  </si>
+  <si>
+    <t>2. Debt-to-assets vs solvency scatterplot.</t>
+  </si>
+  <si>
+    <t>3. Industry-year leverage boxplots.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Larger firms often weather shocks better due to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>cash reserves and credit access</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Smaller firms face higher default risk; comparing groups reveals </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>structural resilience</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Your dataset includes </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>total_assets_eur</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (for size grouping) and profitability ratios (for performance outcomes).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">It investigates </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>heterogeneity within the corporate sector</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">It completes the analysis: profitability (Q1), capital structure (Q2), </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>firm heterogeneity</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (Q3).</t>
+    </r>
+  </si>
+  <si>
+    <t>It provides policy-relevant insights (e.g., SMEs need more support).</t>
+  </si>
+  <si>
+    <t>1. Line plots: EBIT margin and ROA by firm size over time.</t>
+  </si>
+  <si>
+    <t>2. Boxplots: profitability distribution by size and year.</t>
+  </si>
+  <si>
+    <t>3. Scatter: log(total assets) vs EBIT margin with smooth trend.</t>
+  </si>
+  <si>
+    <t>Q2</t>
+  </si>
+  <si>
+    <t>Q3</t>
+  </si>
+  <si>
+    <t>1. Time trends of average leverage indicators
+2. Scatter: leverage vs solvency (are highly levered firms less solvent?)
+3. Boxplots of debt_to_assets by industry, faceted by year</t>
+  </si>
+  <si>
+    <t>1. Profitability by firm size over time
+2. Boxplots of EBIT margin by size within each year
+3. Size–profitability gradient (log assets vs EBIT margin)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -143,13 +796,32 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="8">
@@ -253,16 +925,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -274,18 +953,35 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -602,7 +1298,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A64E804-F5A6-4CE4-9FE3-AFA5E5C714EE}">
   <dimension ref="B2:J23"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="1.3984375" customWidth="1"/>
     <col min="2" max="2" width="13.73046875" bestFit="1" customWidth="1"/>
@@ -615,56 +1311,56 @@
     <col min="9" max="9" width="12.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B2" s="4" t="s">
+    <row r="2" spans="2:10">
+      <c r="B2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="7"/>
-    </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="9" t="s">
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="10"/>
+    </row>
+    <row r="3" spans="2:10">
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="H3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I3" s="9" t="s">
+      <c r="I3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="J3" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B4" s="2" t="s">
+    <row r="4" spans="2:10">
+      <c r="B4" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="3" t="s">
         <v>24</v>
       </c>
       <c r="E4" s="1" t="s">
@@ -676,10 +1372,10 @@
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B5" s="2"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="11"/>
+    <row r="5" spans="2:10">
+      <c r="B5" s="11"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="4"/>
       <c r="E5" s="1" t="s">
         <v>9</v>
       </c>
@@ -689,10 +1385,10 @@
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B6" s="2"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="11"/>
+    <row r="6" spans="2:10">
+      <c r="B6" s="11"/>
+      <c r="C6" s="12"/>
+      <c r="D6" s="4"/>
       <c r="E6" s="1" t="s">
         <v>10</v>
       </c>
@@ -702,10 +1398,10 @@
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B7" s="2"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="12"/>
+    <row r="7" spans="2:10">
+      <c r="B7" s="11"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="5"/>
       <c r="E7" s="1" t="s">
         <v>11</v>
       </c>
@@ -715,14 +1411,14 @@
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B8" s="2" t="s">
+    <row r="8" spans="2:10">
+      <c r="B8" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="3" t="s">
         <v>25</v>
       </c>
       <c r="E8" s="1" t="s">
@@ -734,10 +1430,10 @@
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B9" s="2"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="11"/>
+    <row r="9" spans="2:10">
+      <c r="B9" s="11"/>
+      <c r="C9" s="12"/>
+      <c r="D9" s="4"/>
       <c r="E9" s="1" t="s">
         <v>9</v>
       </c>
@@ -747,10 +1443,10 @@
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B10" s="2"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="11"/>
+    <row r="10" spans="2:10">
+      <c r="B10" s="11"/>
+      <c r="C10" s="12"/>
+      <c r="D10" s="4"/>
       <c r="E10" s="1" t="s">
         <v>10</v>
       </c>
@@ -760,10 +1456,10 @@
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
     </row>
-    <row r="11" spans="2:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B11" s="2"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="12"/>
+    <row r="11" spans="2:10" ht="25.5" customHeight="1">
+      <c r="B11" s="11"/>
+      <c r="C11" s="12"/>
+      <c r="D11" s="5"/>
       <c r="E11" s="1" t="s">
         <v>11</v>
       </c>
@@ -773,14 +1469,14 @@
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B12" s="2" t="s">
+    <row r="12" spans="2:10">
+      <c r="B12" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="3" t="s">
         <v>26</v>
       </c>
       <c r="E12" s="1" t="s">
@@ -792,10 +1488,10 @@
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B13" s="2"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="11"/>
+    <row r="13" spans="2:10">
+      <c r="B13" s="11"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="4"/>
       <c r="E13" s="1" t="s">
         <v>9</v>
       </c>
@@ -805,10 +1501,10 @@
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
     </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B14" s="2"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="11"/>
+    <row r="14" spans="2:10">
+      <c r="B14" s="11"/>
+      <c r="C14" s="12"/>
+      <c r="D14" s="4"/>
       <c r="E14" s="1" t="s">
         <v>10</v>
       </c>
@@ -818,10 +1514,10 @@
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
     </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B15" s="2"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="12"/>
+    <row r="15" spans="2:10">
+      <c r="B15" s="11"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="5"/>
       <c r="E15" s="1" t="s">
         <v>11</v>
       </c>
@@ -831,14 +1527,14 @@
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
     </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B16" s="2" t="s">
+    <row r="16" spans="2:10">
+      <c r="B16" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="3" t="s">
         <v>27</v>
       </c>
       <c r="E16" s="1" t="s">
@@ -850,10 +1546,10 @@
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
     </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B17" s="2"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="11"/>
+    <row r="17" spans="2:10">
+      <c r="B17" s="11"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="4"/>
       <c r="E17" s="1" t="s">
         <v>9</v>
       </c>
@@ -863,10 +1559,10 @@
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
     </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B18" s="2"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="11"/>
+    <row r="18" spans="2:10">
+      <c r="B18" s="11"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="4"/>
       <c r="E18" s="1" t="s">
         <v>10</v>
       </c>
@@ -876,10 +1572,10 @@
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
     </row>
-    <row r="19" spans="2:10" ht="25.15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B19" s="2"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="12"/>
+    <row r="19" spans="2:10" ht="25.15" customHeight="1">
+      <c r="B19" s="11"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="5"/>
       <c r="E19" s="1" t="s">
         <v>11</v>
       </c>
@@ -889,14 +1585,14 @@
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
     </row>
-    <row r="20" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B20" s="2" t="s">
+    <row r="20" spans="2:10">
+      <c r="B20" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="3" t="s">
         <v>28</v>
       </c>
       <c r="E20" s="1" t="s">
@@ -908,10 +1604,10 @@
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
     </row>
-    <row r="21" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B21" s="2"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="11"/>
+    <row r="21" spans="2:10">
+      <c r="B21" s="11"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="4"/>
       <c r="E21" s="1" t="s">
         <v>9</v>
       </c>
@@ -921,10 +1617,10 @@
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
     </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B22" s="2"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="11"/>
+    <row r="22" spans="2:10">
+      <c r="B22" s="11"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="4"/>
       <c r="E22" s="1" t="s">
         <v>10</v>
       </c>
@@ -934,10 +1630,10 @@
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
     </row>
-    <row r="23" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B23" s="2"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="12"/>
+    <row r="23" spans="2:10">
+      <c r="B23" s="11"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="5"/>
       <c r="E23" s="1" t="s">
         <v>11</v>
       </c>
@@ -949,14 +1645,6 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="D16:D19"/>
-    <mergeCell ref="D20:D23"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="F2:J2"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="D4:D7"/>
-    <mergeCell ref="D8:D11"/>
-    <mergeCell ref="D12:D15"/>
     <mergeCell ref="B16:B19"/>
     <mergeCell ref="C16:C19"/>
     <mergeCell ref="C20:C23"/>
@@ -969,6 +1657,450 @@
     <mergeCell ref="C12:C15"/>
     <mergeCell ref="B8:B11"/>
     <mergeCell ref="B12:B15"/>
+    <mergeCell ref="D16:D19"/>
+    <mergeCell ref="D20:D23"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="F2:J2"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="D4:D7"/>
+    <mergeCell ref="D8:D11"/>
+    <mergeCell ref="D12:D15"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75A18CDB-CB7F-4CC2-ACA1-6486E5275781}">
+  <dimension ref="B2:H82"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="2" max="2" width="10.86328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="22.46484375" customWidth="1"/>
+    <col min="6" max="6" width="33.1328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:8" ht="28.5">
+      <c r="B2" s="13"/>
+      <c r="C2" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="13" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" ht="85.5">
+      <c r="B3" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" s="14"/>
+      <c r="F3" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="G3" s="13"/>
+      <c r="H3" s="21" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8" ht="85.5">
+      <c r="B4" s="4"/>
+      <c r="C4" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="G4" s="13"/>
+      <c r="H4" s="22" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" ht="85.5">
+      <c r="B5" s="5"/>
+      <c r="C5" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="G5" s="13"/>
+      <c r="H5" s="22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8">
+      <c r="B6" s="16"/>
+    </row>
+    <row r="7" spans="2:8">
+      <c r="F7" s="20" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8">
+      <c r="B8" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="F8" s="17" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8">
+      <c r="B9" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="F9" s="18"/>
+    </row>
+    <row r="10" spans="2:8">
+      <c r="B10" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="F10" s="18" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8">
+      <c r="B11" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="F11" s="18"/>
+    </row>
+    <row r="12" spans="2:8">
+      <c r="B12" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="F12" s="18" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8">
+      <c r="B13" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="F13" s="18"/>
+    </row>
+    <row r="14" spans="2:8">
+      <c r="B14" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="F14" s="18" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8">
+      <c r="B15" s="15" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8">
+      <c r="B16" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="F16" s="17" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6">
+      <c r="B17" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="F17" s="18"/>
+    </row>
+    <row r="18" spans="2:6">
+      <c r="B18" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="F18" s="18" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6">
+      <c r="B19" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="F19" s="18"/>
+    </row>
+    <row r="20" spans="2:6">
+      <c r="B20" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="F20" s="18" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6">
+      <c r="B21" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="F21" s="18"/>
+    </row>
+    <row r="22" spans="2:6">
+      <c r="B22" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="F22" s="18" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6">
+      <c r="B23" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="F23" s="19" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6">
+      <c r="B24" s="15" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6">
+      <c r="B25" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="F25" s="17" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6">
+      <c r="F26" s="18"/>
+    </row>
+    <row r="27" spans="2:6">
+      <c r="F27" s="18" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6">
+      <c r="F28" s="18"/>
+    </row>
+    <row r="29" spans="2:6">
+      <c r="F29" s="18" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6">
+      <c r="F30" s="18"/>
+    </row>
+    <row r="31" spans="2:6">
+      <c r="F31" s="18" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="33" spans="6:6">
+      <c r="F33" s="20" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="34" spans="6:6">
+      <c r="F34" s="17" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="35" spans="6:6">
+      <c r="F35" s="18"/>
+    </row>
+    <row r="36" spans="6:6">
+      <c r="F36" s="18" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="37" spans="6:6">
+      <c r="F37" s="18"/>
+    </row>
+    <row r="38" spans="6:6">
+      <c r="F38" s="18" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="39" spans="6:6">
+      <c r="F39" s="18"/>
+    </row>
+    <row r="40" spans="6:6">
+      <c r="F40" s="18" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="41" spans="6:6">
+      <c r="F41" s="19" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="43" spans="6:6">
+      <c r="F43" s="17" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="44" spans="6:6">
+      <c r="F44" s="18"/>
+    </row>
+    <row r="45" spans="6:6">
+      <c r="F45" s="18" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="46" spans="6:6">
+      <c r="F46" s="18"/>
+    </row>
+    <row r="47" spans="6:6">
+      <c r="F47" s="18" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="48" spans="6:6">
+      <c r="F48" s="18"/>
+    </row>
+    <row r="49" spans="6:6">
+      <c r="F49" s="18" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="51" spans="6:6">
+      <c r="F51" s="17" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="52" spans="6:6">
+      <c r="F52" s="18"/>
+    </row>
+    <row r="53" spans="6:6">
+      <c r="F53" s="18" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="54" spans="6:6">
+      <c r="F54" s="18"/>
+    </row>
+    <row r="55" spans="6:6">
+      <c r="F55" s="18" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="56" spans="6:6">
+      <c r="F56" s="18"/>
+    </row>
+    <row r="57" spans="6:6">
+      <c r="F57" s="18" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="59" spans="6:6">
+      <c r="F59" s="20" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="60" spans="6:6">
+      <c r="F60" s="17" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="61" spans="6:6">
+      <c r="F61" s="18"/>
+    </row>
+    <row r="62" spans="6:6">
+      <c r="F62" s="18" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="63" spans="6:6">
+      <c r="F63" s="18"/>
+    </row>
+    <row r="64" spans="6:6">
+      <c r="F64" s="18" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="65" spans="6:6">
+      <c r="F65" s="18"/>
+    </row>
+    <row r="66" spans="6:6">
+      <c r="F66" s="18" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="68" spans="6:6">
+      <c r="F68" s="17" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="69" spans="6:6">
+      <c r="F69" s="18"/>
+    </row>
+    <row r="70" spans="6:6">
+      <c r="F70" s="18" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="71" spans="6:6">
+      <c r="F71" s="18"/>
+    </row>
+    <row r="72" spans="6:6">
+      <c r="F72" s="18" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="73" spans="6:6">
+      <c r="F73" s="18"/>
+    </row>
+    <row r="74" spans="6:6">
+      <c r="F74" s="18" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="76" spans="6:6">
+      <c r="F76" s="17" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="77" spans="6:6">
+      <c r="F77" s="18"/>
+    </row>
+    <row r="78" spans="6:6">
+      <c r="F78" s="18" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="79" spans="6:6">
+      <c r="F79" s="18"/>
+    </row>
+    <row r="80" spans="6:6">
+      <c r="F80" s="18" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="81" spans="6:6">
+      <c r="F81" s="18"/>
+    </row>
+    <row r="82" spans="6:6">
+      <c r="F82" s="18" t="s">
+        <v>89</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B3:B5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
finalising the sub-questions to answer the primary question
</commit_message>
<xml_diff>
--- a/Project Plan.xlsx
+++ b/Project Plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Semester 2\ETC5521\Project 1\project-part-1-p1-wallaby\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F590E7D2-60E1-4B99-8A20-BF4FE8E552E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79FABB6D-EE25-4850-824A-1EEF0EF9551F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{08FA5D9B-BDCD-4B0C-BBC1-0603E7BA2D97}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{08FA5D9B-BDCD-4B0C-BBC1-0603E7BA2D97}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Plan" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="99">
   <si>
     <t>Section</t>
   </si>
@@ -774,6 +774,23 @@
     <t>1. Profitability by firm size over time
 2. Boxplots of EBIT margin by size within each year
 3. Size–profitability gradient (log assets vs EBIT margin)</t>
+  </si>
+  <si>
+    <t>How did firm size influence financial resilience during the pandemic period (2020–2022)?</t>
+  </si>
+  <si>
+    <t>How did the fundamental relationship between corporate liquidity and profitability evolve and fracture within industries during the pandemic?</t>
+  </si>
+  <si>
+    <t>1. A feasts feature scatter plot.
+2. A Scagnostics metrics timeline.
+3. A "normal" vs "abnormal" industry comparison scatter plot.</t>
+  </si>
+  <si>
+    <t>Member</t>
+  </si>
+  <si>
+    <t>ROA (%) (data31070) ,Current ratio (data31105)  , company_id</t>
   </si>
 </sst>
 </file>
@@ -925,48 +942,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -977,11 +963,62 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1312,31 +1349,31 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
-      <c r="I2" s="9"/>
-      <c r="J2" s="10"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="19"/>
     </row>
     <row r="3" spans="2:10">
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
       <c r="F3" s="2" t="s">
         <v>12</v>
       </c>
@@ -1353,72 +1390,80 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="2:10">
+    <row r="4" spans="2:10" s="5" customFormat="1" ht="20.350000000000001" customHeight="1">
       <c r="B4" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-    </row>
-    <row r="5" spans="2:10">
+      <c r="F4" s="23" t="s">
+        <v>32</v>
+      </c>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
+      <c r="I4" s="24"/>
+      <c r="J4" s="25"/>
+    </row>
+    <row r="5" spans="2:10" s="5" customFormat="1" ht="31.15" customHeight="1">
       <c r="B5" s="11"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="1" t="s">
+      <c r="C5" s="11"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-    </row>
-    <row r="6" spans="2:10">
+      <c r="F5" s="23" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" s="24"/>
+      <c r="H5" s="24"/>
+      <c r="I5" s="24"/>
+      <c r="J5" s="25"/>
+    </row>
+    <row r="6" spans="2:10" s="5" customFormat="1" ht="30.75" customHeight="1">
       <c r="B6" s="11"/>
-      <c r="C6" s="12"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="1" t="s">
+      <c r="C6" s="11"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-    </row>
-    <row r="7" spans="2:10">
+      <c r="F6" s="23" t="s">
+        <v>94</v>
+      </c>
+      <c r="G6" s="24"/>
+      <c r="H6" s="24"/>
+      <c r="I6" s="24"/>
+      <c r="J6" s="25"/>
+    </row>
+    <row r="7" spans="2:10" s="5" customFormat="1" ht="31.9" customHeight="1">
       <c r="B7" s="11"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="1" t="s">
+      <c r="C7" s="11"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
+      <c r="F7" s="23" t="s">
+        <v>95</v>
+      </c>
+      <c r="G7" s="24"/>
+      <c r="H7" s="24"/>
+      <c r="I7" s="24"/>
+      <c r="J7" s="25"/>
     </row>
     <row r="8" spans="2:10">
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="14" t="s">
         <v>25</v>
       </c>
       <c r="E8" s="1" t="s">
@@ -1431,9 +1476,9 @@
       <c r="J8" s="1"/>
     </row>
     <row r="9" spans="2:10">
-      <c r="B9" s="11"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="4"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="15"/>
       <c r="E9" s="1" t="s">
         <v>9</v>
       </c>
@@ -1444,9 +1489,9 @@
       <c r="J9" s="1"/>
     </row>
     <row r="10" spans="2:10">
-      <c r="B10" s="11"/>
-      <c r="C10" s="12"/>
-      <c r="D10" s="4"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="15"/>
       <c r="E10" s="1" t="s">
         <v>10</v>
       </c>
@@ -1457,9 +1502,9 @@
       <c r="J10" s="1"/>
     </row>
     <row r="11" spans="2:10" ht="25.5" customHeight="1">
-      <c r="B11" s="11"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="5"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="16"/>
       <c r="E11" s="1" t="s">
         <v>11</v>
       </c>
@@ -1470,13 +1515,13 @@
       <c r="J11" s="1"/>
     </row>
     <row r="12" spans="2:10">
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="C12" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="14" t="s">
         <v>26</v>
       </c>
       <c r="E12" s="1" t="s">
@@ -1489,9 +1534,9 @@
       <c r="J12" s="1"/>
     </row>
     <row r="13" spans="2:10">
-      <c r="B13" s="11"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="4"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="15"/>
       <c r="E13" s="1" t="s">
         <v>9</v>
       </c>
@@ -1502,9 +1547,9 @@
       <c r="J13" s="1"/>
     </row>
     <row r="14" spans="2:10">
-      <c r="B14" s="11"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="4"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="15"/>
       <c r="E14" s="1" t="s">
         <v>10</v>
       </c>
@@ -1515,9 +1560,9 @@
       <c r="J14" s="1"/>
     </row>
     <row r="15" spans="2:10">
-      <c r="B15" s="11"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="5"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="16"/>
       <c r="E15" s="1" t="s">
         <v>11</v>
       </c>
@@ -1528,13 +1573,13 @@
       <c r="J15" s="1"/>
     </row>
     <row r="16" spans="2:10">
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="12" t="s">
+      <c r="C16" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="14" t="s">
         <v>27</v>
       </c>
       <c r="E16" s="1" t="s">
@@ -1547,9 +1592,9 @@
       <c r="J16" s="1"/>
     </row>
     <row r="17" spans="2:10">
-      <c r="B17" s="11"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="4"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="15"/>
       <c r="E17" s="1" t="s">
         <v>9</v>
       </c>
@@ -1560,9 +1605,9 @@
       <c r="J17" s="1"/>
     </row>
     <row r="18" spans="2:10">
-      <c r="B18" s="11"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="4"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="15"/>
       <c r="E18" s="1" t="s">
         <v>10</v>
       </c>
@@ -1573,9 +1618,9 @@
       <c r="J18" s="1"/>
     </row>
     <row r="19" spans="2:10" ht="25.15" customHeight="1">
-      <c r="B19" s="11"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="5"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="16"/>
       <c r="E19" s="1" t="s">
         <v>11</v>
       </c>
@@ -1586,13 +1631,13 @@
       <c r="J19" s="1"/>
     </row>
     <row r="20" spans="2:10">
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C20" s="12" t="s">
+      <c r="C20" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="14" t="s">
         <v>28</v>
       </c>
       <c r="E20" s="1" t="s">
@@ -1605,9 +1650,9 @@
       <c r="J20" s="1"/>
     </row>
     <row r="21" spans="2:10">
-      <c r="B21" s="11"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="4"/>
+      <c r="B21" s="10"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="15"/>
       <c r="E21" s="1" t="s">
         <v>9</v>
       </c>
@@ -1618,9 +1663,9 @@
       <c r="J21" s="1"/>
     </row>
     <row r="22" spans="2:10">
-      <c r="B22" s="11"/>
-      <c r="C22" s="12"/>
-      <c r="D22" s="4"/>
+      <c r="B22" s="10"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="15"/>
       <c r="E22" s="1" t="s">
         <v>10</v>
       </c>
@@ -1631,9 +1676,9 @@
       <c r="J22" s="1"/>
     </row>
     <row r="23" spans="2:10">
-      <c r="B23" s="11"/>
-      <c r="C23" s="12"/>
-      <c r="D23" s="5"/>
+      <c r="B23" s="10"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="16"/>
       <c r="E23" s="1" t="s">
         <v>11</v>
       </c>
@@ -1644,7 +1689,19 @@
       <c r="J23" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="24">
+    <mergeCell ref="D16:D19"/>
+    <mergeCell ref="D20:D23"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="F2:J2"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="D4:D7"/>
+    <mergeCell ref="D8:D11"/>
+    <mergeCell ref="D12:D15"/>
+    <mergeCell ref="F4:J4"/>
+    <mergeCell ref="F5:J5"/>
+    <mergeCell ref="F6:J6"/>
+    <mergeCell ref="F7:J7"/>
     <mergeCell ref="B16:B19"/>
     <mergeCell ref="C16:C19"/>
     <mergeCell ref="C20:C23"/>
@@ -1657,14 +1714,6 @@
     <mergeCell ref="C12:C15"/>
     <mergeCell ref="B8:B11"/>
     <mergeCell ref="B12:B15"/>
-    <mergeCell ref="D16:D19"/>
-    <mergeCell ref="D20:D23"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="F2:J2"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="D4:D7"/>
-    <mergeCell ref="D8:D11"/>
-    <mergeCell ref="D12:D15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1672,7 +1721,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75A18CDB-CB7F-4CC2-ACA1-6486E5275781}">
-  <dimension ref="B2:H82"/>
+  <dimension ref="B2:H83"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="2" max="2" width="10.86328125" bestFit="1" customWidth="1"/>
@@ -1681,420 +1730,446 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" ht="28.5">
-      <c r="B2" s="13"/>
-      <c r="C2" s="13" t="s">
+      <c r="B2" s="4"/>
+      <c r="C2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="G2" s="4" t="s">
         <v>21</v>
       </c>
+      <c r="H2" s="22" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="3" spans="2:8" ht="85.5">
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="14"/>
-      <c r="F3" s="13" t="s">
+      <c r="E3" s="4"/>
+      <c r="F3" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="G3" s="13"/>
-      <c r="H3" s="21" t="s">
+      <c r="G3" s="4"/>
+      <c r="H3" s="4" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="4" spans="2:8" ht="85.5">
-      <c r="B4" s="4"/>
-      <c r="C4" s="14" t="s">
+      <c r="B4" s="15"/>
+      <c r="C4" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13" t="s">
+      <c r="E4" s="4"/>
+      <c r="F4" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="G4" s="13"/>
-      <c r="H4" s="22" t="s">
+      <c r="G4" s="4"/>
+      <c r="H4" s="4" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5" spans="2:8" ht="85.5">
-      <c r="B5" s="5"/>
-      <c r="C5" s="14" t="s">
+      <c r="B5" s="15"/>
+      <c r="C5" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13" t="s">
+      <c r="E5" s="21"/>
+      <c r="F5" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="G5" s="13"/>
-      <c r="H5" s="22" t="s">
+      <c r="G5" s="21"/>
+      <c r="H5" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="2:8">
-      <c r="B6" s="16"/>
+    <row r="6" spans="2:8" ht="85.5">
+      <c r="B6" s="4"/>
+      <c r="C6" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="E6" s="26"/>
+      <c r="F6" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="G6" s="26"/>
+      <c r="H6" s="26" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="7" spans="2:8">
-      <c r="F7" s="20" t="s">
+      <c r="B7" s="27"/>
+      <c r="C7" s="20"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="28"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="28"/>
+      <c r="H7" s="28"/>
+    </row>
+    <row r="8" spans="2:8">
+      <c r="F8" s="9" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="8" spans="2:8">
-      <c r="B8" s="15" t="s">
+    <row r="9" spans="2:8">
+      <c r="B9" t="s">
         <v>38</v>
       </c>
-      <c r="F8" s="17" t="s">
+      <c r="F9" s="6" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="9" spans="2:8">
-      <c r="B9" s="15" t="s">
+    <row r="10" spans="2:8">
+      <c r="B10" t="s">
         <v>39</v>
       </c>
-      <c r="F9" s="18"/>
-    </row>
-    <row r="10" spans="2:8">
-      <c r="B10" s="15" t="s">
+      <c r="F10" s="7"/>
+    </row>
+    <row r="11" spans="2:8">
+      <c r="B11" t="s">
         <v>40</v>
       </c>
-      <c r="F10" s="18" t="s">
+      <c r="F11" s="7" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="11" spans="2:8">
-      <c r="B11" s="15" t="s">
+    <row r="12" spans="2:8">
+      <c r="B12" t="s">
         <v>52</v>
       </c>
-      <c r="F11" s="18"/>
-    </row>
-    <row r="12" spans="2:8">
-      <c r="B12" s="15" t="s">
+      <c r="F12" s="7"/>
+    </row>
+    <row r="13" spans="2:8">
+      <c r="B13" t="s">
         <v>43</v>
       </c>
-      <c r="F12" s="18" t="s">
+      <c r="F13" s="7" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="13" spans="2:8">
-      <c r="B13" s="15" t="s">
+    <row r="14" spans="2:8">
+      <c r="B14" t="s">
         <v>44</v>
       </c>
-      <c r="F13" s="18"/>
-    </row>
-    <row r="14" spans="2:8">
-      <c r="B14" s="15" t="s">
+      <c r="F14" s="7"/>
+    </row>
+    <row r="15" spans="2:8">
+      <c r="B15" t="s">
         <v>45</v>
       </c>
-      <c r="F14" s="18" t="s">
+      <c r="F15" s="7" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="15" spans="2:8">
-      <c r="B15" s="15" t="s">
+    <row r="16" spans="2:8">
+      <c r="B16" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="16" spans="2:8">
-      <c r="B16" s="15" t="s">
+    <row r="17" spans="2:6">
+      <c r="B17" t="s">
         <v>35</v>
       </c>
-      <c r="F16" s="17" t="s">
+      <c r="F17" s="6" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="17" spans="2:6">
-      <c r="B17" s="15" t="s">
+    <row r="18" spans="2:6">
+      <c r="B18" t="s">
         <v>47</v>
       </c>
-      <c r="F17" s="18"/>
-    </row>
-    <row r="18" spans="2:6">
-      <c r="B18" s="15" t="s">
+      <c r="F18" s="7"/>
+    </row>
+    <row r="19" spans="2:6">
+      <c r="B19" t="s">
         <v>36</v>
       </c>
-      <c r="F18" s="18" t="s">
+      <c r="F19" s="7" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="19" spans="2:6">
-      <c r="B19" s="15" t="s">
+    <row r="20" spans="2:6">
+      <c r="B20" t="s">
         <v>48</v>
       </c>
-      <c r="F19" s="18"/>
-    </row>
-    <row r="20" spans="2:6">
-      <c r="B20" s="15" t="s">
+      <c r="F20" s="7"/>
+    </row>
+    <row r="21" spans="2:6">
+      <c r="B21" t="s">
         <v>49</v>
       </c>
-      <c r="F20" s="18" t="s">
+      <c r="F21" s="7" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="21" spans="2:6">
-      <c r="B21" s="15" t="s">
+    <row r="22" spans="2:6">
+      <c r="B22" t="s">
         <v>50</v>
       </c>
-      <c r="F21" s="18"/>
-    </row>
-    <row r="22" spans="2:6">
-      <c r="B22" s="15" t="s">
+      <c r="F22" s="7"/>
+    </row>
+    <row r="23" spans="2:6">
+      <c r="B23" t="s">
         <v>51</v>
       </c>
-      <c r="F22" s="18" t="s">
+      <c r="F23" s="7" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="23" spans="2:6">
-      <c r="B23" s="15" t="s">
+    <row r="24" spans="2:6">
+      <c r="B24" t="s">
         <v>41</v>
       </c>
-      <c r="F23" s="19" t="s">
+      <c r="F24" s="8" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="24" spans="2:6">
-      <c r="B24" s="15" t="s">
+    <row r="25" spans="2:6">
+      <c r="B25" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="25" spans="2:6">
-      <c r="B25" s="15" t="s">
+    <row r="26" spans="2:6">
+      <c r="B26" t="s">
         <v>37</v>
       </c>
-      <c r="F25" s="17" t="s">
+      <c r="F26" s="6" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="26" spans="2:6">
-      <c r="F26" s="18"/>
-    </row>
     <row r="27" spans="2:6">
-      <c r="F27" s="18" t="s">
+      <c r="F27" s="7"/>
+    </row>
+    <row r="28" spans="2:6">
+      <c r="F28" s="7" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="28" spans="2:6">
-      <c r="F28" s="18"/>
-    </row>
     <row r="29" spans="2:6">
-      <c r="F29" s="18" t="s">
+      <c r="F29" s="7"/>
+    </row>
+    <row r="30" spans="2:6">
+      <c r="F30" s="7" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="30" spans="2:6">
-      <c r="F30" s="18"/>
-    </row>
     <row r="31" spans="2:6">
-      <c r="F31" s="18" t="s">
+      <c r="F31" s="7"/>
+    </row>
+    <row r="32" spans="2:6">
+      <c r="F32" s="7" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="33" spans="6:6">
-      <c r="F33" s="20" t="s">
+    <row r="34" spans="6:6">
+      <c r="F34" s="9" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="34" spans="6:6">
-      <c r="F34" s="17" t="s">
+    <row r="35" spans="6:6">
+      <c r="F35" s="6" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="35" spans="6:6">
-      <c r="F35" s="18"/>
-    </row>
     <row r="36" spans="6:6">
-      <c r="F36" s="18" t="s">
+      <c r="F36" s="7"/>
+    </row>
+    <row r="37" spans="6:6">
+      <c r="F37" s="7" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="37" spans="6:6">
-      <c r="F37" s="18"/>
-    </row>
     <row r="38" spans="6:6">
-      <c r="F38" s="18" t="s">
+      <c r="F38" s="7"/>
+    </row>
+    <row r="39" spans="6:6">
+      <c r="F39" s="7" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="39" spans="6:6">
-      <c r="F39" s="18"/>
-    </row>
     <row r="40" spans="6:6">
-      <c r="F40" s="18" t="s">
+      <c r="F40" s="7"/>
+    </row>
+    <row r="41" spans="6:6">
+      <c r="F41" s="7" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="41" spans="6:6">
-      <c r="F41" s="19" t="s">
+    <row r="42" spans="6:6">
+      <c r="F42" s="8" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="43" spans="6:6">
-      <c r="F43" s="17" t="s">
+    <row r="44" spans="6:6">
+      <c r="F44" s="6" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="44" spans="6:6">
-      <c r="F44" s="18"/>
-    </row>
     <row r="45" spans="6:6">
-      <c r="F45" s="18" t="s">
+      <c r="F45" s="7"/>
+    </row>
+    <row r="46" spans="6:6">
+      <c r="F46" s="7" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="46" spans="6:6">
-      <c r="F46" s="18"/>
-    </row>
     <row r="47" spans="6:6">
-      <c r="F47" s="18" t="s">
+      <c r="F47" s="7"/>
+    </row>
+    <row r="48" spans="6:6">
+      <c r="F48" s="7" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="48" spans="6:6">
-      <c r="F48" s="18"/>
-    </row>
     <row r="49" spans="6:6">
-      <c r="F49" s="18" t="s">
+      <c r="F49" s="7"/>
+    </row>
+    <row r="50" spans="6:6">
+      <c r="F50" s="7" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="51" spans="6:6">
-      <c r="F51" s="17" t="s">
+    <row r="52" spans="6:6">
+      <c r="F52" s="6" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="52" spans="6:6">
-      <c r="F52" s="18"/>
-    </row>
     <row r="53" spans="6:6">
-      <c r="F53" s="18" t="s">
+      <c r="F53" s="7"/>
+    </row>
+    <row r="54" spans="6:6">
+      <c r="F54" s="7" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="54" spans="6:6">
-      <c r="F54" s="18"/>
-    </row>
     <row r="55" spans="6:6">
-      <c r="F55" s="18" t="s">
+      <c r="F55" s="7"/>
+    </row>
+    <row r="56" spans="6:6">
+      <c r="F56" s="7" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="56" spans="6:6">
-      <c r="F56" s="18"/>
-    </row>
     <row r="57" spans="6:6">
-      <c r="F57" s="18" t="s">
+      <c r="F57" s="7"/>
+    </row>
+    <row r="58" spans="6:6">
+      <c r="F58" s="7" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="59" spans="6:6">
-      <c r="F59" s="20" t="s">
+    <row r="60" spans="6:6">
+      <c r="F60" s="9" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="60" spans="6:6">
-      <c r="F60" s="17" t="s">
+    <row r="61" spans="6:6">
+      <c r="F61" s="6" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="61" spans="6:6">
-      <c r="F61" s="18"/>
-    </row>
     <row r="62" spans="6:6">
-      <c r="F62" s="18" t="s">
+      <c r="F62" s="7"/>
+    </row>
+    <row r="63" spans="6:6">
+      <c r="F63" s="7" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="63" spans="6:6">
-      <c r="F63" s="18"/>
-    </row>
     <row r="64" spans="6:6">
-      <c r="F64" s="18" t="s">
+      <c r="F64" s="7"/>
+    </row>
+    <row r="65" spans="6:6">
+      <c r="F65" s="7" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="65" spans="6:6">
-      <c r="F65" s="18"/>
-    </row>
     <row r="66" spans="6:6">
-      <c r="F66" s="18" t="s">
+      <c r="F66" s="7"/>
+    </row>
+    <row r="67" spans="6:6">
+      <c r="F67" s="7" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="68" spans="6:6">
-      <c r="F68" s="17" t="s">
+    <row r="69" spans="6:6">
+      <c r="F69" s="6" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="69" spans="6:6">
-      <c r="F69" s="18"/>
-    </row>
     <row r="70" spans="6:6">
-      <c r="F70" s="18" t="s">
+      <c r="F70" s="7"/>
+    </row>
+    <row r="71" spans="6:6">
+      <c r="F71" s="7" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="71" spans="6:6">
-      <c r="F71" s="18"/>
-    </row>
     <row r="72" spans="6:6">
-      <c r="F72" s="18" t="s">
+      <c r="F72" s="7"/>
+    </row>
+    <row r="73" spans="6:6">
+      <c r="F73" s="7" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="73" spans="6:6">
-      <c r="F73" s="18"/>
-    </row>
     <row r="74" spans="6:6">
-      <c r="F74" s="18" t="s">
+      <c r="F74" s="7"/>
+    </row>
+    <row r="75" spans="6:6">
+      <c r="F75" s="7" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="76" spans="6:6">
-      <c r="F76" s="17" t="s">
+    <row r="77" spans="6:6">
+      <c r="F77" s="6" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="77" spans="6:6">
-      <c r="F77" s="18"/>
-    </row>
     <row r="78" spans="6:6">
-      <c r="F78" s="18" t="s">
+      <c r="F78" s="7"/>
+    </row>
+    <row r="79" spans="6:6">
+      <c r="F79" s="7" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="79" spans="6:6">
-      <c r="F79" s="18"/>
-    </row>
     <row r="80" spans="6:6">
-      <c r="F80" s="18" t="s">
+      <c r="F80" s="7"/>
+    </row>
+    <row r="81" spans="6:6">
+      <c r="F81" s="7" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="81" spans="6:6">
-      <c r="F81" s="18"/>
-    </row>
     <row r="82" spans="6:6">
-      <c r="F82" s="18" t="s">
+      <c r="F82" s="7"/>
+    </row>
+    <row r="83" spans="6:6">
+      <c r="F83" s="7" t="s">
         <v>89</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Change the project plan and select the columns.
</commit_message>
<xml_diff>
--- a/Project Plan.xlsx
+++ b/Project Plan.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Semester 2\ETC5521\Project 1\project-part-1-p1-wallaby\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\10354\monash_git\5521\project1\project-part-1-p1-wallaby\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79FABB6D-EE25-4850-824A-1EEF0EF9551F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0503039-8688-4A85-B77D-B08A083CDC29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{08FA5D9B-BDCD-4B0C-BBC1-0603E7BA2D97}"/>
+    <workbookView xWindow="11685" yWindow="945" windowWidth="10380" windowHeight="13568" xr2:uid="{08FA5D9B-BDCD-4B0C-BBC1-0603E7BA2D97}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Plan" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="100">
   <si>
     <t>Section</t>
   </si>
@@ -220,7 +220,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -230,7 +230,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -246,7 +246,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -256,7 +256,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -272,7 +272,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -282,7 +282,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -304,7 +304,7 @@
         <i/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -314,7 +314,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -332,7 +332,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -350,7 +350,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -368,7 +368,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -386,7 +386,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -417,7 +417,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -427,7 +427,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -443,7 +443,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -453,7 +453,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -464,7 +464,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -474,7 +474,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -492,7 +492,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -510,7 +510,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -528,7 +528,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -546,7 +546,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -562,7 +562,7 @@
         <i/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -572,7 +572,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -588,7 +588,7 @@
         <i/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -598,7 +598,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -629,7 +629,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -639,7 +639,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -655,7 +655,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -665,7 +665,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -688,7 +688,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -704,7 +704,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -714,7 +714,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -730,7 +730,7 @@
         <i/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -740,7 +740,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -791,17 +791,21 @@
   </si>
   <si>
     <t>ROA (%) (data31070) ,Current ratio (data31105)  , company_id</t>
+  </si>
+  <si>
+    <t>Jingyi</t>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -809,7 +813,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -817,7 +821,7 @@
       <i/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -825,6 +829,20 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="3">
@@ -841,7 +859,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -938,11 +956,22 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -963,17 +992,17 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -984,6 +1013,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -992,15 +1027,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1012,17 +1038,17 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1038,7 +1064,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 主题​​">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1335,7 +1361,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A64E804-F5A6-4CE4-9FE3-AFA5E5C714EE}">
   <dimension ref="B2:J23"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.9"/>
   <cols>
     <col min="1" max="1" width="1.3984375" customWidth="1"/>
     <col min="2" max="2" width="13.73046875" bestFit="1" customWidth="1"/>
@@ -1349,31 +1375,31 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10">
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="F2" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-      <c r="J2" s="19"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="21"/>
     </row>
     <row r="3" spans="2:10">
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
       <c r="F3" s="2" t="s">
         <v>12</v>
       </c>
@@ -1391,10 +1417,10 @@
       </c>
     </row>
     <row r="4" spans="2:10" s="5" customFormat="1" ht="20.350000000000001" customHeight="1">
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="26" t="s">
         <v>18</v>
       </c>
       <c r="D4" s="14" t="s">
@@ -1403,64 +1429,64 @@
       <c r="E4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="23" t="s">
+      <c r="F4" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="G4" s="24"/>
-      <c r="H4" s="24"/>
-      <c r="I4" s="24"/>
-      <c r="J4" s="25"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
+      <c r="I4" s="23"/>
+      <c r="J4" s="24"/>
     </row>
     <row r="5" spans="2:10" s="5" customFormat="1" ht="31.15" customHeight="1">
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
+      <c r="B5" s="26"/>
+      <c r="C5" s="26"/>
       <c r="D5" s="15"/>
       <c r="E5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" s="23"/>
+      <c r="H5" s="23"/>
+      <c r="I5" s="23"/>
+      <c r="J5" s="24"/>
+    </row>
+    <row r="6" spans="2:10" s="5" customFormat="1" ht="30.75" customHeight="1">
+      <c r="B6" s="26"/>
+      <c r="C6" s="26"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="23" t="s">
-        <v>30</v>
-      </c>
-      <c r="G5" s="24"/>
-      <c r="H5" s="24"/>
-      <c r="I5" s="24"/>
-      <c r="J5" s="25"/>
-    </row>
-    <row r="6" spans="2:10" s="5" customFormat="1" ht="30.75" customHeight="1">
-      <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F6" s="23" t="s">
+      <c r="F6" s="22" t="s">
         <v>94</v>
       </c>
-      <c r="G6" s="24"/>
-      <c r="H6" s="24"/>
-      <c r="I6" s="24"/>
-      <c r="J6" s="25"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="23"/>
+      <c r="I6" s="23"/>
+      <c r="J6" s="24"/>
     </row>
     <row r="7" spans="2:10" s="5" customFormat="1" ht="31.9" customHeight="1">
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
+      <c r="B7" s="26"/>
+      <c r="C7" s="26"/>
       <c r="D7" s="16"/>
       <c r="E7" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="F7" s="22" t="s">
         <v>95</v>
       </c>
-      <c r="G7" s="24"/>
-      <c r="H7" s="24"/>
-      <c r="I7" s="24"/>
-      <c r="J7" s="25"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="24"/>
     </row>
     <row r="8" spans="2:10">
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="26" t="s">
         <v>16</v>
       </c>
       <c r="D8" s="14" t="s">
@@ -1476,8 +1502,8 @@
       <c r="J8" s="1"/>
     </row>
     <row r="9" spans="2:10">
-      <c r="B9" s="10"/>
-      <c r="C9" s="11"/>
+      <c r="B9" s="25"/>
+      <c r="C9" s="26"/>
       <c r="D9" s="15"/>
       <c r="E9" s="1" t="s">
         <v>9</v>
@@ -1488,9 +1514,9 @@
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
     </row>
-    <row r="10" spans="2:10">
-      <c r="B10" s="10"/>
-      <c r="C10" s="11"/>
+    <row r="10" spans="2:10" ht="13.9" customHeight="1">
+      <c r="B10" s="25"/>
+      <c r="C10" s="26"/>
       <c r="D10" s="15"/>
       <c r="E10" s="1" t="s">
         <v>10</v>
@@ -1502,8 +1528,8 @@
       <c r="J10" s="1"/>
     </row>
     <row r="11" spans="2:10" ht="25.5" customHeight="1">
-      <c r="B11" s="10"/>
-      <c r="C11" s="11"/>
+      <c r="B11" s="25"/>
+      <c r="C11" s="26"/>
       <c r="D11" s="16"/>
       <c r="E11" s="1" t="s">
         <v>11</v>
@@ -1515,10 +1541,10 @@
       <c r="J11" s="1"/>
     </row>
     <row r="12" spans="2:10">
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="26" t="s">
         <v>17</v>
       </c>
       <c r="D12" s="14" t="s">
@@ -1534,8 +1560,8 @@
       <c r="J12" s="1"/>
     </row>
     <row r="13" spans="2:10">
-      <c r="B13" s="10"/>
-      <c r="C13" s="11"/>
+      <c r="B13" s="25"/>
+      <c r="C13" s="26"/>
       <c r="D13" s="15"/>
       <c r="E13" s="1" t="s">
         <v>9</v>
@@ -1547,8 +1573,8 @@
       <c r="J13" s="1"/>
     </row>
     <row r="14" spans="2:10">
-      <c r="B14" s="10"/>
-      <c r="C14" s="11"/>
+      <c r="B14" s="25"/>
+      <c r="C14" s="26"/>
       <c r="D14" s="15"/>
       <c r="E14" s="1" t="s">
         <v>10</v>
@@ -1560,8 +1586,8 @@
       <c r="J14" s="1"/>
     </row>
     <row r="15" spans="2:10">
-      <c r="B15" s="10"/>
-      <c r="C15" s="11"/>
+      <c r="B15" s="25"/>
+      <c r="C15" s="26"/>
       <c r="D15" s="16"/>
       <c r="E15" s="1" t="s">
         <v>11</v>
@@ -1573,10 +1599,10 @@
       <c r="J15" s="1"/>
     </row>
     <row r="16" spans="2:10">
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="C16" s="26" t="s">
         <v>19</v>
       </c>
       <c r="D16" s="14" t="s">
@@ -1592,8 +1618,8 @@
       <c r="J16" s="1"/>
     </row>
     <row r="17" spans="2:10">
-      <c r="B17" s="10"/>
-      <c r="C17" s="11"/>
+      <c r="B17" s="25"/>
+      <c r="C17" s="26"/>
       <c r="D17" s="15"/>
       <c r="E17" s="1" t="s">
         <v>9</v>
@@ -1605,8 +1631,8 @@
       <c r="J17" s="1"/>
     </row>
     <row r="18" spans="2:10">
-      <c r="B18" s="10"/>
-      <c r="C18" s="11"/>
+      <c r="B18" s="25"/>
+      <c r="C18" s="26"/>
       <c r="D18" s="15"/>
       <c r="E18" s="1" t="s">
         <v>10</v>
@@ -1618,8 +1644,8 @@
       <c r="J18" s="1"/>
     </row>
     <row r="19" spans="2:10" ht="25.15" customHeight="1">
-      <c r="B19" s="10"/>
-      <c r="C19" s="11"/>
+      <c r="B19" s="25"/>
+      <c r="C19" s="26"/>
       <c r="D19" s="16"/>
       <c r="E19" s="1" t="s">
         <v>11</v>
@@ -1631,10 +1657,10 @@
       <c r="J19" s="1"/>
     </row>
     <row r="20" spans="2:10">
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="26" t="s">
         <v>20</v>
       </c>
       <c r="D20" s="14" t="s">
@@ -1650,8 +1676,8 @@
       <c r="J20" s="1"/>
     </row>
     <row r="21" spans="2:10">
-      <c r="B21" s="10"/>
-      <c r="C21" s="11"/>
+      <c r="B21" s="25"/>
+      <c r="C21" s="26"/>
       <c r="D21" s="15"/>
       <c r="E21" s="1" t="s">
         <v>9</v>
@@ -1663,8 +1689,8 @@
       <c r="J21" s="1"/>
     </row>
     <row r="22" spans="2:10">
-      <c r="B22" s="10"/>
-      <c r="C22" s="11"/>
+      <c r="B22" s="25"/>
+      <c r="C22" s="26"/>
       <c r="D22" s="15"/>
       <c r="E22" s="1" t="s">
         <v>10</v>
@@ -1676,8 +1702,8 @@
       <c r="J22" s="1"/>
     </row>
     <row r="23" spans="2:10">
-      <c r="B23" s="10"/>
-      <c r="C23" s="11"/>
+      <c r="B23" s="25"/>
+      <c r="C23" s="26"/>
       <c r="D23" s="16"/>
       <c r="E23" s="1" t="s">
         <v>11</v>
@@ -1690,6 +1716,18 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="B16:B19"/>
+    <mergeCell ref="C16:C19"/>
+    <mergeCell ref="C20:C23"/>
+    <mergeCell ref="B20:B23"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="B4:B7"/>
+    <mergeCell ref="C4:C7"/>
+    <mergeCell ref="C8:C11"/>
+    <mergeCell ref="C12:C15"/>
+    <mergeCell ref="B8:B11"/>
+    <mergeCell ref="B12:B15"/>
     <mergeCell ref="D16:D19"/>
     <mergeCell ref="D20:D23"/>
     <mergeCell ref="E2:E3"/>
@@ -1702,19 +1740,8 @@
     <mergeCell ref="F5:J5"/>
     <mergeCell ref="F6:J6"/>
     <mergeCell ref="F7:J7"/>
-    <mergeCell ref="B16:B19"/>
-    <mergeCell ref="C16:C19"/>
-    <mergeCell ref="C20:C23"/>
-    <mergeCell ref="B20:B23"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="B4:B7"/>
-    <mergeCell ref="C4:C7"/>
-    <mergeCell ref="C8:C11"/>
-    <mergeCell ref="C12:C15"/>
-    <mergeCell ref="B8:B11"/>
-    <mergeCell ref="B12:B15"/>
   </mergeCells>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1722,14 +1749,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75A18CDB-CB7F-4CC2-ACA1-6486E5275781}">
   <dimension ref="B2:H83"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.9"/>
   <cols>
     <col min="2" max="2" width="10.86328125" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="22.46484375" customWidth="1"/>
     <col min="6" max="6" width="33.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" ht="28.5">
+    <row r="2" spans="2:8" ht="27.75">
       <c r="B2" s="4"/>
       <c r="C2" s="4" t="s">
         <v>4</v>
@@ -1746,11 +1773,11 @@
       <c r="G2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H2" s="22" t="s">
+      <c r="H2" s="4" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="2:8" ht="85.5">
+    <row r="3" spans="2:8" ht="83.25">
       <c r="B3" s="14" t="s">
         <v>29</v>
       </c>
@@ -1769,7 +1796,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="2:8" ht="85.5">
+    <row r="4" spans="2:8" ht="83.25">
       <c r="B4" s="15"/>
       <c r="C4" s="4" t="s">
         <v>30</v>
@@ -1786,48 +1813,48 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="2:8" ht="85.5">
+    <row r="5" spans="2:8" ht="83.25">
       <c r="B5" s="15"/>
-      <c r="C5" s="21" t="s">
+      <c r="C5" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="21" t="s">
+      <c r="D5" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="E5" s="21"/>
-      <c r="F5" s="21" t="s">
+      <c r="E5" s="11"/>
+      <c r="F5" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="G5" s="21"/>
+      <c r="G5" s="11"/>
       <c r="H5" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="2:8" ht="85.5">
+    <row r="6" spans="2:8" ht="83.25">
       <c r="B6" s="4"/>
-      <c r="C6" s="22" t="s">
+      <c r="C6" s="4" t="s">
         <v>95</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="E6" s="26"/>
+      <c r="E6" s="12"/>
       <c r="F6" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="G6" s="26"/>
-      <c r="H6" s="26" t="s">
+      <c r="G6" s="12"/>
+      <c r="H6" s="12" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="7" spans="2:8">
-      <c r="B7" s="27"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="27"/>
-      <c r="E7" s="28"/>
-      <c r="F7" s="27"/>
-      <c r="G7" s="28"/>
-      <c r="H7" s="28"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
     </row>
     <row r="8" spans="2:8">
       <c r="F8" s="9" t="s">
@@ -2177,6 +2204,7 @@
   <mergeCells count="1">
     <mergeCell ref="B3:B5"/>
   </mergeCells>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Create a branch -Jing, change plan and write the work diary.
</commit_message>
<xml_diff>
--- a/Project Plan.xlsx
+++ b/Project Plan.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Semester 2\ETC5521\Project 1\project-part-1-p1-wallaby\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\10354\monash_git\5521\project1\project-part-1-p1-wallaby\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79FABB6D-EE25-4850-824A-1EEF0EF9551F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0503039-8688-4A85-B77D-B08A083CDC29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{08FA5D9B-BDCD-4B0C-BBC1-0603E7BA2D97}"/>
+    <workbookView xWindow="11685" yWindow="945" windowWidth="10380" windowHeight="13568" xr2:uid="{08FA5D9B-BDCD-4B0C-BBC1-0603E7BA2D97}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Plan" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="100">
   <si>
     <t>Section</t>
   </si>
@@ -220,7 +220,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -230,7 +230,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -246,7 +246,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -256,7 +256,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -272,7 +272,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -282,7 +282,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -304,7 +304,7 @@
         <i/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -314,7 +314,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -332,7 +332,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -350,7 +350,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -368,7 +368,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -386,7 +386,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -417,7 +417,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -427,7 +427,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -443,7 +443,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -453,7 +453,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -464,7 +464,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -474,7 +474,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -492,7 +492,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -510,7 +510,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -528,7 +528,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -546,7 +546,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -562,7 +562,7 @@
         <i/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -572,7 +572,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -588,7 +588,7 @@
         <i/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -598,7 +598,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -629,7 +629,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -639,7 +639,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -655,7 +655,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -665,7 +665,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -688,7 +688,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -704,7 +704,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -714,7 +714,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -730,7 +730,7 @@
         <i/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -740,7 +740,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="等线"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -791,17 +791,21 @@
   </si>
   <si>
     <t>ROA (%) (data31070) ,Current ratio (data31105)  , company_id</t>
+  </si>
+  <si>
+    <t>Jingyi</t>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -809,7 +813,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -817,7 +821,7 @@
       <i/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -825,6 +829,20 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="3">
@@ -841,7 +859,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -938,11 +956,22 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -963,17 +992,17 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -984,6 +1013,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -992,15 +1027,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1012,17 +1038,17 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1038,7 +1064,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 主题​​">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1335,7 +1361,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A64E804-F5A6-4CE4-9FE3-AFA5E5C714EE}">
   <dimension ref="B2:J23"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.9"/>
   <cols>
     <col min="1" max="1" width="1.3984375" customWidth="1"/>
     <col min="2" max="2" width="13.73046875" bestFit="1" customWidth="1"/>
@@ -1349,31 +1375,31 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10">
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="F2" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-      <c r="J2" s="19"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="21"/>
     </row>
     <row r="3" spans="2:10">
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
       <c r="F3" s="2" t="s">
         <v>12</v>
       </c>
@@ -1391,10 +1417,10 @@
       </c>
     </row>
     <row r="4" spans="2:10" s="5" customFormat="1" ht="20.350000000000001" customHeight="1">
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="26" t="s">
         <v>18</v>
       </c>
       <c r="D4" s="14" t="s">
@@ -1403,64 +1429,64 @@
       <c r="E4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="23" t="s">
+      <c r="F4" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="G4" s="24"/>
-      <c r="H4" s="24"/>
-      <c r="I4" s="24"/>
-      <c r="J4" s="25"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
+      <c r="I4" s="23"/>
+      <c r="J4" s="24"/>
     </row>
     <row r="5" spans="2:10" s="5" customFormat="1" ht="31.15" customHeight="1">
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
+      <c r="B5" s="26"/>
+      <c r="C5" s="26"/>
       <c r="D5" s="15"/>
       <c r="E5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" s="23"/>
+      <c r="H5" s="23"/>
+      <c r="I5" s="23"/>
+      <c r="J5" s="24"/>
+    </row>
+    <row r="6" spans="2:10" s="5" customFormat="1" ht="30.75" customHeight="1">
+      <c r="B6" s="26"/>
+      <c r="C6" s="26"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="23" t="s">
-        <v>30</v>
-      </c>
-      <c r="G5" s="24"/>
-      <c r="H5" s="24"/>
-      <c r="I5" s="24"/>
-      <c r="J5" s="25"/>
-    </row>
-    <row r="6" spans="2:10" s="5" customFormat="1" ht="30.75" customHeight="1">
-      <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F6" s="23" t="s">
+      <c r="F6" s="22" t="s">
         <v>94</v>
       </c>
-      <c r="G6" s="24"/>
-      <c r="H6" s="24"/>
-      <c r="I6" s="24"/>
-      <c r="J6" s="25"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="23"/>
+      <c r="I6" s="23"/>
+      <c r="J6" s="24"/>
     </row>
     <row r="7" spans="2:10" s="5" customFormat="1" ht="31.9" customHeight="1">
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
+      <c r="B7" s="26"/>
+      <c r="C7" s="26"/>
       <c r="D7" s="16"/>
       <c r="E7" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="F7" s="22" t="s">
         <v>95</v>
       </c>
-      <c r="G7" s="24"/>
-      <c r="H7" s="24"/>
-      <c r="I7" s="24"/>
-      <c r="J7" s="25"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="24"/>
     </row>
     <row r="8" spans="2:10">
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="26" t="s">
         <v>16</v>
       </c>
       <c r="D8" s="14" t="s">
@@ -1476,8 +1502,8 @@
       <c r="J8" s="1"/>
     </row>
     <row r="9" spans="2:10">
-      <c r="B9" s="10"/>
-      <c r="C9" s="11"/>
+      <c r="B9" s="25"/>
+      <c r="C9" s="26"/>
       <c r="D9" s="15"/>
       <c r="E9" s="1" t="s">
         <v>9</v>
@@ -1488,9 +1514,9 @@
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
     </row>
-    <row r="10" spans="2:10">
-      <c r="B10" s="10"/>
-      <c r="C10" s="11"/>
+    <row r="10" spans="2:10" ht="13.9" customHeight="1">
+      <c r="B10" s="25"/>
+      <c r="C10" s="26"/>
       <c r="D10" s="15"/>
       <c r="E10" s="1" t="s">
         <v>10</v>
@@ -1502,8 +1528,8 @@
       <c r="J10" s="1"/>
     </row>
     <row r="11" spans="2:10" ht="25.5" customHeight="1">
-      <c r="B11" s="10"/>
-      <c r="C11" s="11"/>
+      <c r="B11" s="25"/>
+      <c r="C11" s="26"/>
       <c r="D11" s="16"/>
       <c r="E11" s="1" t="s">
         <v>11</v>
@@ -1515,10 +1541,10 @@
       <c r="J11" s="1"/>
     </row>
     <row r="12" spans="2:10">
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="26" t="s">
         <v>17</v>
       </c>
       <c r="D12" s="14" t="s">
@@ -1534,8 +1560,8 @@
       <c r="J12" s="1"/>
     </row>
     <row r="13" spans="2:10">
-      <c r="B13" s="10"/>
-      <c r="C13" s="11"/>
+      <c r="B13" s="25"/>
+      <c r="C13" s="26"/>
       <c r="D13" s="15"/>
       <c r="E13" s="1" t="s">
         <v>9</v>
@@ -1547,8 +1573,8 @@
       <c r="J13" s="1"/>
     </row>
     <row r="14" spans="2:10">
-      <c r="B14" s="10"/>
-      <c r="C14" s="11"/>
+      <c r="B14" s="25"/>
+      <c r="C14" s="26"/>
       <c r="D14" s="15"/>
       <c r="E14" s="1" t="s">
         <v>10</v>
@@ -1560,8 +1586,8 @@
       <c r="J14" s="1"/>
     </row>
     <row r="15" spans="2:10">
-      <c r="B15" s="10"/>
-      <c r="C15" s="11"/>
+      <c r="B15" s="25"/>
+      <c r="C15" s="26"/>
       <c r="D15" s="16"/>
       <c r="E15" s="1" t="s">
         <v>11</v>
@@ -1573,10 +1599,10 @@
       <c r="J15" s="1"/>
     </row>
     <row r="16" spans="2:10">
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="C16" s="26" t="s">
         <v>19</v>
       </c>
       <c r="D16" s="14" t="s">
@@ -1592,8 +1618,8 @@
       <c r="J16" s="1"/>
     </row>
     <row r="17" spans="2:10">
-      <c r="B17" s="10"/>
-      <c r="C17" s="11"/>
+      <c r="B17" s="25"/>
+      <c r="C17" s="26"/>
       <c r="D17" s="15"/>
       <c r="E17" s="1" t="s">
         <v>9</v>
@@ -1605,8 +1631,8 @@
       <c r="J17" s="1"/>
     </row>
     <row r="18" spans="2:10">
-      <c r="B18" s="10"/>
-      <c r="C18" s="11"/>
+      <c r="B18" s="25"/>
+      <c r="C18" s="26"/>
       <c r="D18" s="15"/>
       <c r="E18" s="1" t="s">
         <v>10</v>
@@ -1618,8 +1644,8 @@
       <c r="J18" s="1"/>
     </row>
     <row r="19" spans="2:10" ht="25.15" customHeight="1">
-      <c r="B19" s="10"/>
-      <c r="C19" s="11"/>
+      <c r="B19" s="25"/>
+      <c r="C19" s="26"/>
       <c r="D19" s="16"/>
       <c r="E19" s="1" t="s">
         <v>11</v>
@@ -1631,10 +1657,10 @@
       <c r="J19" s="1"/>
     </row>
     <row r="20" spans="2:10">
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="26" t="s">
         <v>20</v>
       </c>
       <c r="D20" s="14" t="s">
@@ -1650,8 +1676,8 @@
       <c r="J20" s="1"/>
     </row>
     <row r="21" spans="2:10">
-      <c r="B21" s="10"/>
-      <c r="C21" s="11"/>
+      <c r="B21" s="25"/>
+      <c r="C21" s="26"/>
       <c r="D21" s="15"/>
       <c r="E21" s="1" t="s">
         <v>9</v>
@@ -1663,8 +1689,8 @@
       <c r="J21" s="1"/>
     </row>
     <row r="22" spans="2:10">
-      <c r="B22" s="10"/>
-      <c r="C22" s="11"/>
+      <c r="B22" s="25"/>
+      <c r="C22" s="26"/>
       <c r="D22" s="15"/>
       <c r="E22" s="1" t="s">
         <v>10</v>
@@ -1676,8 +1702,8 @@
       <c r="J22" s="1"/>
     </row>
     <row r="23" spans="2:10">
-      <c r="B23" s="10"/>
-      <c r="C23" s="11"/>
+      <c r="B23" s="25"/>
+      <c r="C23" s="26"/>
       <c r="D23" s="16"/>
       <c r="E23" s="1" t="s">
         <v>11</v>
@@ -1690,6 +1716,18 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="B16:B19"/>
+    <mergeCell ref="C16:C19"/>
+    <mergeCell ref="C20:C23"/>
+    <mergeCell ref="B20:B23"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="B4:B7"/>
+    <mergeCell ref="C4:C7"/>
+    <mergeCell ref="C8:C11"/>
+    <mergeCell ref="C12:C15"/>
+    <mergeCell ref="B8:B11"/>
+    <mergeCell ref="B12:B15"/>
     <mergeCell ref="D16:D19"/>
     <mergeCell ref="D20:D23"/>
     <mergeCell ref="E2:E3"/>
@@ -1702,19 +1740,8 @@
     <mergeCell ref="F5:J5"/>
     <mergeCell ref="F6:J6"/>
     <mergeCell ref="F7:J7"/>
-    <mergeCell ref="B16:B19"/>
-    <mergeCell ref="C16:C19"/>
-    <mergeCell ref="C20:C23"/>
-    <mergeCell ref="B20:B23"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="B4:B7"/>
-    <mergeCell ref="C4:C7"/>
-    <mergeCell ref="C8:C11"/>
-    <mergeCell ref="C12:C15"/>
-    <mergeCell ref="B8:B11"/>
-    <mergeCell ref="B12:B15"/>
   </mergeCells>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1722,14 +1749,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75A18CDB-CB7F-4CC2-ACA1-6486E5275781}">
   <dimension ref="B2:H83"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.9"/>
   <cols>
     <col min="2" max="2" width="10.86328125" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="22.46484375" customWidth="1"/>
     <col min="6" max="6" width="33.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" ht="28.5">
+    <row r="2" spans="2:8" ht="27.75">
       <c r="B2" s="4"/>
       <c r="C2" s="4" t="s">
         <v>4</v>
@@ -1746,11 +1773,11 @@
       <c r="G2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H2" s="22" t="s">
+      <c r="H2" s="4" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="2:8" ht="85.5">
+    <row r="3" spans="2:8" ht="83.25">
       <c r="B3" s="14" t="s">
         <v>29</v>
       </c>
@@ -1769,7 +1796,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="2:8" ht="85.5">
+    <row r="4" spans="2:8" ht="83.25">
       <c r="B4" s="15"/>
       <c r="C4" s="4" t="s">
         <v>30</v>
@@ -1786,48 +1813,48 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="2:8" ht="85.5">
+    <row r="5" spans="2:8" ht="83.25">
       <c r="B5" s="15"/>
-      <c r="C5" s="21" t="s">
+      <c r="C5" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="21" t="s">
+      <c r="D5" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="E5" s="21"/>
-      <c r="F5" s="21" t="s">
+      <c r="E5" s="11"/>
+      <c r="F5" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="G5" s="21"/>
+      <c r="G5" s="11"/>
       <c r="H5" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="2:8" ht="85.5">
+    <row r="6" spans="2:8" ht="83.25">
       <c r="B6" s="4"/>
-      <c r="C6" s="22" t="s">
+      <c r="C6" s="4" t="s">
         <v>95</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="E6" s="26"/>
+      <c r="E6" s="12"/>
       <c r="F6" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="G6" s="26"/>
-      <c r="H6" s="26" t="s">
+      <c r="G6" s="12"/>
+      <c r="H6" s="12" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="7" spans="2:8">
-      <c r="B7" s="27"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="27"/>
-      <c r="E7" s="28"/>
-      <c r="F7" s="27"/>
-      <c r="G7" s="28"/>
-      <c r="H7" s="28"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
     </row>
     <row r="8" spans="2:8">
       <c r="F8" s="9" t="s">
@@ -2177,6 +2204,7 @@
   <mergeCells count="1">
     <mergeCell ref="B3:B5"/>
   </mergeCells>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
creating data description table
</commit_message>
<xml_diff>
--- a/Project Plan.xlsx
+++ b/Project Plan.xlsx
@@ -5,16 +5,17 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\10354\monash_git\5521\project1\project-part-1-p1-wallaby\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Semester 2\ETC5521\Project 1\project-part-1-p1-wallaby\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0503039-8688-4A85-B77D-B08A083CDC29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAD0521C-EA03-4FBC-8B23-36689C979B3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11685" yWindow="945" windowWidth="10380" windowHeight="13568" xr2:uid="{08FA5D9B-BDCD-4B0C-BBC1-0603E7BA2D97}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="2" xr2:uid="{08FA5D9B-BDCD-4B0C-BBC1-0603E7BA2D97}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Plan" sheetId="1" r:id="rId1"/>
     <sheet name="Team Analysis" sheetId="2" r:id="rId2"/>
+    <sheet name="Data Description" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="198">
   <si>
     <t>Section</t>
   </si>
@@ -220,7 +221,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -230,7 +231,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -246,7 +247,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -256,7 +257,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -272,7 +273,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -282,7 +283,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -304,7 +305,7 @@
         <i/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -314,7 +315,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -332,7 +333,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -350,7 +351,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -368,7 +369,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -386,7 +387,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -417,7 +418,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -427,7 +428,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -443,7 +444,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -453,7 +454,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -464,7 +465,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -474,7 +475,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -492,7 +493,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -510,7 +511,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -528,7 +529,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -546,7 +547,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -562,7 +563,7 @@
         <i/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -572,7 +573,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -588,7 +589,7 @@
         <i/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -598,7 +599,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -629,7 +630,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -639,7 +640,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -655,7 +656,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -665,7 +666,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -688,7 +689,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -704,7 +705,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -714,7 +715,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -730,7 +731,7 @@
         <i/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -740,7 +741,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="等线"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -795,17 +796,323 @@
   <si>
     <t>Jingyi</t>
     <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Column Name</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Data Type</t>
+  </si>
+  <si>
+    <t>company_id</t>
+  </si>
+  <si>
+    <t>Unique company identifier (Bureau van Dijk ID).</t>
+  </si>
+  <si>
+    <t>character</t>
+  </si>
+  <si>
+    <t>BvD ID Number (os_id_number)</t>
+  </si>
+  <si>
+    <t>company_name</t>
+  </si>
+  <si>
+    <t>Registered company name (label).</t>
+  </si>
+  <si>
+    <t>Company Name (name)</t>
+  </si>
+  <si>
+    <t>fy_end_date</t>
+  </si>
+  <si>
+    <t>Company fiscal year-end date for the account.</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>Company Fiscal Year End Date (closdate)</t>
+  </si>
+  <si>
+    <t>fy_year</t>
+  </si>
+  <si>
+    <t>Year extracted from fiscal year-end date.</t>
+  </si>
+  <si>
+    <t>integer</t>
+  </si>
+  <si>
+    <t>acct_year</t>
+  </si>
+  <si>
+    <t>Reporting year label carried from file name/field.</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>country</t>
+  </si>
+  <si>
+    <t>Country of head office.</t>
+  </si>
+  <si>
+    <t>Country (country)</t>
+  </si>
+  <si>
+    <t>city</t>
+  </si>
+  <si>
+    <t>City of head office.</t>
+  </si>
+  <si>
+    <t>CITY - City (city)</t>
+  </si>
+  <si>
+    <t>consolidation_code</t>
+  </si>
+  <si>
+    <t>Consolidation scope of the accounts (e.g., C1/C2/U1/U2).</t>
+  </si>
+  <si>
+    <t>Consolidation Code (consol_code)</t>
+  </si>
+  <si>
+    <t>nace_code</t>
+  </si>
+  <si>
+    <t>NACE core code (EU industry classification).</t>
+  </si>
+  <si>
+    <t>NACE Rev 1, Core Code (cnacecd)</t>
+  </si>
+  <si>
+    <t>icb_code</t>
+  </si>
+  <si>
+    <t>ICB industry classification code.</t>
+  </si>
+  <si>
+    <t>Industrial Classification Benchmark (icb)</t>
+  </si>
+  <si>
+    <t>sic_code</t>
+  </si>
+  <si>
+    <t>US SIC core code.</t>
+  </si>
+  <si>
+    <t>US SIC, Core Code (csicuscde)</t>
+  </si>
+  <si>
+    <t>total_assets_eur</t>
+  </si>
+  <si>
+    <t>Total assets (EUR).</t>
+  </si>
+  <si>
+    <t>numeric</t>
+  </si>
+  <si>
+    <t>Total Assets (data13077)</t>
+  </si>
+  <si>
+    <t>total_liabilities_eur</t>
+  </si>
+  <si>
+    <t>Total liabilities and debt (EUR).</t>
+  </si>
+  <si>
+    <t>Total Liabilities and Debt (data14022)</t>
+  </si>
+  <si>
+    <t>total_equity_eur</t>
+  </si>
+  <si>
+    <t>Total shareholders’ equity (EUR).</t>
+  </si>
+  <si>
+    <t>Total Shareholders Equity (data14041)</t>
+  </si>
+  <si>
+    <t>total_revenue_eur</t>
+  </si>
+  <si>
+    <t>Total revenues / operating revenue (EUR).</t>
+  </si>
+  <si>
+    <t>Total revenues (data13004)</t>
+  </si>
+  <si>
+    <t>net_sales_eur</t>
+  </si>
+  <si>
+    <t>Net sales (EUR).</t>
+  </si>
+  <si>
+    <t>Net sales (data13002)</t>
+  </si>
+  <si>
+    <t>gross_sales_eur</t>
+  </si>
+  <si>
+    <t>Gross sales (EUR).</t>
+  </si>
+  <si>
+    <t>Gross sales (data13000)</t>
+  </si>
+  <si>
+    <t>net_income_eur</t>
+  </si>
+  <si>
+    <t>Net income (EUR).</t>
+  </si>
+  <si>
+    <t>Net Income / Starting Line (data15500)</t>
+  </si>
+  <si>
+    <t>ebit_margin_pct</t>
+  </si>
+  <si>
+    <t>EBIT margin (% of sales/revenue).</t>
+  </si>
+  <si>
+    <t>EBIT Margin (%) (data31055)</t>
+  </si>
+  <si>
+    <t>ebitda_margin_pct</t>
+  </si>
+  <si>
+    <t>EBITDA margin (% of sales/revenue).</t>
+  </si>
+  <si>
+    <t>EBITDA Margin (%) (data31060)</t>
+  </si>
+  <si>
+    <t>roa_pct</t>
+  </si>
+  <si>
+    <t>Return on total assets (%).</t>
+  </si>
+  <si>
+    <t>Return on Total Assets (%) (data31015)</t>
+  </si>
+  <si>
+    <t>roe_pct</t>
+  </si>
+  <si>
+    <t>Return on equity (%).</t>
+  </si>
+  <si>
+    <t>ROE (%) (data31065)</t>
+  </si>
+  <si>
+    <t>net_assets_turnover</t>
+  </si>
+  <si>
+    <t>Net assets turnover (times).</t>
+  </si>
+  <si>
+    <t>Net Assets Turnover (data31225)</t>
+  </si>
+  <si>
+    <t>stock_turnover</t>
+  </si>
+  <si>
+    <t>Stock / inventory turnover (times).</t>
+  </si>
+  <si>
+    <t>Stock Turnover (data31220)</t>
+  </si>
+  <si>
+    <t>solvency_pct</t>
+  </si>
+  <si>
+    <t>Solvency ratio (%).</t>
+  </si>
+  <si>
+    <t>Solvency ratio (%) (data31310)</t>
+  </si>
+  <si>
+    <t>gearing_pct</t>
+  </si>
+  <si>
+    <t>Gearing ratio (%).</t>
+  </si>
+  <si>
+    <t>Gearing (%) (data31315)</t>
+  </si>
+  <si>
+    <t>current_ratio</t>
+  </si>
+  <si>
+    <t>Current ratio (times).</t>
+  </si>
+  <si>
+    <t>Current ratio (data31105)</t>
+  </si>
+  <si>
+    <t>liquidity_ratio</t>
+  </si>
+  <si>
+    <t>Liquidity / quick ratio (times).</t>
+  </si>
+  <si>
+    <t>Liquidity ratio (data31110)</t>
+  </si>
+  <si>
+    <t>shareholders_liq_pct</t>
+  </si>
+  <si>
+    <t>Shareholders’ liquidity ratio (%).</t>
+  </si>
+  <si>
+    <t>Shareholders Liquidity ratio (data31305)</t>
+  </si>
+  <si>
+    <t>interest_cover</t>
+  </si>
+  <si>
+    <t>Interest cover (times).</t>
+  </si>
+  <si>
+    <t>Interest Cover (data31115)</t>
+  </si>
+  <si>
+    <r>
+      <t>derived from</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Company Fiscal Year End Date (closdate)</t>
+    </r>
+  </si>
+  <si>
+    <t>Original Name</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -813,7 +1120,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -821,7 +1128,7 @@
       <i/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -832,7 +1139,7 @@
     </font>
     <font>
       <sz val="9"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -843,6 +1150,13 @@
       <name val="等线"/>
       <family val="3"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -971,7 +1285,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1004,6 +1318,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1012,12 +1341,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1037,18 +1360,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1064,7 +1387,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 主题​​">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1361,7 +1684,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A64E804-F5A6-4CE4-9FE3-AFA5E5C714EE}">
   <dimension ref="B2:J23"/>
-  <sheetFormatPr defaultRowHeight="13.9"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="1.3984375" customWidth="1"/>
     <col min="2" max="2" width="13.73046875" bestFit="1" customWidth="1"/>
@@ -1387,13 +1710,13 @@
       <c r="E2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="19" t="s">
+      <c r="F2" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
-      <c r="J2" s="21"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="24"/>
     </row>
     <row r="3" spans="2:10">
       <c r="B3" s="18"/>
@@ -1417,79 +1740,79 @@
       </c>
     </row>
     <row r="4" spans="2:10" s="5" customFormat="1" ht="20.350000000000001" customHeight="1">
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="26" t="s">
+      <c r="C4" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="19" t="s">
         <v>24</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="22" t="s">
+      <c r="F4" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="G4" s="23"/>
-      <c r="H4" s="23"/>
-      <c r="I4" s="23"/>
-      <c r="J4" s="24"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="26"/>
+      <c r="I4" s="26"/>
+      <c r="J4" s="27"/>
     </row>
     <row r="5" spans="2:10" s="5" customFormat="1" ht="31.15" customHeight="1">
-      <c r="B5" s="26"/>
-      <c r="C5" s="26"/>
-      <c r="D5" s="15"/>
+      <c r="B5" s="16"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="20"/>
       <c r="E5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="22" t="s">
+      <c r="F5" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="G5" s="23"/>
-      <c r="H5" s="23"/>
-      <c r="I5" s="23"/>
-      <c r="J5" s="24"/>
+      <c r="G5" s="26"/>
+      <c r="H5" s="26"/>
+      <c r="I5" s="26"/>
+      <c r="J5" s="27"/>
     </row>
     <row r="6" spans="2:10" s="5" customFormat="1" ht="30.75" customHeight="1">
-      <c r="B6" s="26"/>
-      <c r="C6" s="26"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="27" t="s">
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="22" t="s">
+      <c r="F6" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="G6" s="23"/>
-      <c r="H6" s="23"/>
-      <c r="I6" s="23"/>
-      <c r="J6" s="24"/>
+      <c r="G6" s="26"/>
+      <c r="H6" s="26"/>
+      <c r="I6" s="26"/>
+      <c r="J6" s="27"/>
     </row>
     <row r="7" spans="2:10" s="5" customFormat="1" ht="31.9" customHeight="1">
-      <c r="B7" s="26"/>
-      <c r="C7" s="26"/>
-      <c r="D7" s="16"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="21"/>
       <c r="E7" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="F7" s="22" t="s">
+      <c r="F7" s="25" t="s">
         <v>95</v>
       </c>
-      <c r="G7" s="23"/>
-      <c r="H7" s="23"/>
-      <c r="I7" s="23"/>
-      <c r="J7" s="24"/>
+      <c r="G7" s="26"/>
+      <c r="H7" s="26"/>
+      <c r="I7" s="26"/>
+      <c r="J7" s="27"/>
     </row>
     <row r="8" spans="2:10">
-      <c r="B8" s="25" t="s">
+      <c r="B8" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="26" t="s">
+      <c r="C8" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="D8" s="19" t="s">
         <v>25</v>
       </c>
       <c r="E8" s="1" t="s">
@@ -1502,9 +1825,9 @@
       <c r="J8" s="1"/>
     </row>
     <row r="9" spans="2:10">
-      <c r="B9" s="25"/>
-      <c r="C9" s="26"/>
-      <c r="D9" s="15"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="20"/>
       <c r="E9" s="1" t="s">
         <v>9</v>
       </c>
@@ -1515,9 +1838,9 @@
       <c r="J9" s="1"/>
     </row>
     <row r="10" spans="2:10" ht="13.9" customHeight="1">
-      <c r="B10" s="25"/>
-      <c r="C10" s="26"/>
-      <c r="D10" s="15"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="20"/>
       <c r="E10" s="1" t="s">
         <v>10</v>
       </c>
@@ -1528,9 +1851,9 @@
       <c r="J10" s="1"/>
     </row>
     <row r="11" spans="2:10" ht="25.5" customHeight="1">
-      <c r="B11" s="25"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="16"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="21"/>
       <c r="E11" s="1" t="s">
         <v>11</v>
       </c>
@@ -1541,13 +1864,13 @@
       <c r="J11" s="1"/>
     </row>
     <row r="12" spans="2:10">
-      <c r="B12" s="25" t="s">
+      <c r="B12" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="26" t="s">
+      <c r="C12" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="14" t="s">
+      <c r="D12" s="19" t="s">
         <v>26</v>
       </c>
       <c r="E12" s="1" t="s">
@@ -1560,9 +1883,9 @@
       <c r="J12" s="1"/>
     </row>
     <row r="13" spans="2:10">
-      <c r="B13" s="25"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="15"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="20"/>
       <c r="E13" s="1" t="s">
         <v>9</v>
       </c>
@@ -1573,9 +1896,9 @@
       <c r="J13" s="1"/>
     </row>
     <row r="14" spans="2:10">
-      <c r="B14" s="25"/>
-      <c r="C14" s="26"/>
-      <c r="D14" s="15"/>
+      <c r="B14" s="15"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="20"/>
       <c r="E14" s="1" t="s">
         <v>10</v>
       </c>
@@ -1586,9 +1909,9 @@
       <c r="J14" s="1"/>
     </row>
     <row r="15" spans="2:10">
-      <c r="B15" s="25"/>
-      <c r="C15" s="26"/>
-      <c r="D15" s="16"/>
+      <c r="B15" s="15"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="21"/>
       <c r="E15" s="1" t="s">
         <v>11</v>
       </c>
@@ -1599,13 +1922,13 @@
       <c r="J15" s="1"/>
     </row>
     <row r="16" spans="2:10">
-      <c r="B16" s="25" t="s">
+      <c r="B16" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="26" t="s">
+      <c r="C16" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="D16" s="14" t="s">
+      <c r="D16" s="19" t="s">
         <v>27</v>
       </c>
       <c r="E16" s="1" t="s">
@@ -1618,9 +1941,9 @@
       <c r="J16" s="1"/>
     </row>
     <row r="17" spans="2:10">
-      <c r="B17" s="25"/>
-      <c r="C17" s="26"/>
-      <c r="D17" s="15"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="20"/>
       <c r="E17" s="1" t="s">
         <v>9</v>
       </c>
@@ -1631,9 +1954,9 @@
       <c r="J17" s="1"/>
     </row>
     <row r="18" spans="2:10">
-      <c r="B18" s="25"/>
-      <c r="C18" s="26"/>
-      <c r="D18" s="15"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="20"/>
       <c r="E18" s="1" t="s">
         <v>10</v>
       </c>
@@ -1644,9 +1967,9 @@
       <c r="J18" s="1"/>
     </row>
     <row r="19" spans="2:10" ht="25.15" customHeight="1">
-      <c r="B19" s="25"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="16"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="16"/>
+      <c r="D19" s="21"/>
       <c r="E19" s="1" t="s">
         <v>11</v>
       </c>
@@ -1657,13 +1980,13 @@
       <c r="J19" s="1"/>
     </row>
     <row r="20" spans="2:10">
-      <c r="B20" s="25" t="s">
+      <c r="B20" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="C20" s="26" t="s">
+      <c r="C20" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="D20" s="14" t="s">
+      <c r="D20" s="19" t="s">
         <v>28</v>
       </c>
       <c r="E20" s="1" t="s">
@@ -1676,9 +1999,9 @@
       <c r="J20" s="1"/>
     </row>
     <row r="21" spans="2:10">
-      <c r="B21" s="25"/>
-      <c r="C21" s="26"/>
-      <c r="D21" s="15"/>
+      <c r="B21" s="15"/>
+      <c r="C21" s="16"/>
+      <c r="D21" s="20"/>
       <c r="E21" s="1" t="s">
         <v>9</v>
       </c>
@@ -1689,9 +2012,9 @@
       <c r="J21" s="1"/>
     </row>
     <row r="22" spans="2:10">
-      <c r="B22" s="25"/>
-      <c r="C22" s="26"/>
-      <c r="D22" s="15"/>
+      <c r="B22" s="15"/>
+      <c r="C22" s="16"/>
+      <c r="D22" s="20"/>
       <c r="E22" s="1" t="s">
         <v>10</v>
       </c>
@@ -1702,9 +2025,9 @@
       <c r="J22" s="1"/>
     </row>
     <row r="23" spans="2:10">
-      <c r="B23" s="25"/>
-      <c r="C23" s="26"/>
-      <c r="D23" s="16"/>
+      <c r="B23" s="15"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="21"/>
       <c r="E23" s="1" t="s">
         <v>11</v>
       </c>
@@ -1716,6 +2039,18 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="D16:D19"/>
+    <mergeCell ref="D20:D23"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="F2:J2"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="D4:D7"/>
+    <mergeCell ref="D8:D11"/>
+    <mergeCell ref="D12:D15"/>
+    <mergeCell ref="F4:J4"/>
+    <mergeCell ref="F5:J5"/>
+    <mergeCell ref="F6:J6"/>
+    <mergeCell ref="F7:J7"/>
     <mergeCell ref="B16:B19"/>
     <mergeCell ref="C16:C19"/>
     <mergeCell ref="C20:C23"/>
@@ -1728,18 +2063,6 @@
     <mergeCell ref="C12:C15"/>
     <mergeCell ref="B8:B11"/>
     <mergeCell ref="B12:B15"/>
-    <mergeCell ref="D16:D19"/>
-    <mergeCell ref="D20:D23"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="F2:J2"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="D4:D7"/>
-    <mergeCell ref="D8:D11"/>
-    <mergeCell ref="D12:D15"/>
-    <mergeCell ref="F4:J4"/>
-    <mergeCell ref="F5:J5"/>
-    <mergeCell ref="F6:J6"/>
-    <mergeCell ref="F7:J7"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1749,14 +2072,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75A18CDB-CB7F-4CC2-ACA1-6486E5275781}">
   <dimension ref="B2:H83"/>
-  <sheetFormatPr defaultRowHeight="13.9"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="2" max="2" width="10.86328125" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="22.46484375" customWidth="1"/>
     <col min="6" max="6" width="33.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" ht="27.75">
+    <row r="2" spans="2:8" ht="28.5">
       <c r="B2" s="4"/>
       <c r="C2" s="4" t="s">
         <v>4</v>
@@ -1777,8 +2100,8 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="2:8" ht="83.25">
-      <c r="B3" s="14" t="s">
+    <row r="3" spans="2:8" ht="85.5">
+      <c r="B3" s="19" t="s">
         <v>29</v>
       </c>
       <c r="C3" s="4" t="s">
@@ -1796,8 +2119,8 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="2:8" ht="83.25">
-      <c r="B4" s="15"/>
+    <row r="4" spans="2:8" ht="85.5">
+      <c r="B4" s="20"/>
       <c r="C4" s="4" t="s">
         <v>30</v>
       </c>
@@ -1813,8 +2136,8 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="2:8" ht="83.25">
-      <c r="B5" s="15"/>
+    <row r="5" spans="2:8" ht="85.5">
+      <c r="B5" s="20"/>
       <c r="C5" s="11" t="s">
         <v>31</v>
       </c>
@@ -1830,7 +2153,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="2:8" ht="83.25">
+    <row r="6" spans="2:8" ht="85.5">
       <c r="B6" s="4"/>
       <c r="C6" s="4" t="s">
         <v>95</v>
@@ -2207,4 +2530,455 @@
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{386DA283-C632-433B-8FFD-60F2EE5387D7}">
+  <dimension ref="B2:E32"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="2" max="2" width="25.19921875" customWidth="1"/>
+    <col min="3" max="3" width="48.73046875" customWidth="1"/>
+    <col min="4" max="4" width="15.46484375" customWidth="1"/>
+    <col min="5" max="5" width="44.1328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:5">
+      <c r="B2" s="28" t="s">
+        <v>100</v>
+      </c>
+      <c r="C2" s="28" t="s">
+        <v>101</v>
+      </c>
+      <c r="D2" s="28" t="s">
+        <v>102</v>
+      </c>
+      <c r="E2" s="28" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5">
+      <c r="B3" s="29" t="s">
+        <v>103</v>
+      </c>
+      <c r="C3" s="29" t="s">
+        <v>104</v>
+      </c>
+      <c r="D3" s="29" t="s">
+        <v>105</v>
+      </c>
+      <c r="E3" s="29" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5">
+      <c r="B4" s="29" t="s">
+        <v>107</v>
+      </c>
+      <c r="C4" s="29" t="s">
+        <v>108</v>
+      </c>
+      <c r="D4" s="29" t="s">
+        <v>105</v>
+      </c>
+      <c r="E4" s="29" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5">
+      <c r="B5" s="29" t="s">
+        <v>110</v>
+      </c>
+      <c r="C5" s="29" t="s">
+        <v>111</v>
+      </c>
+      <c r="D5" s="29" t="s">
+        <v>112</v>
+      </c>
+      <c r="E5" s="29" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5">
+      <c r="B6" s="29" t="s">
+        <v>114</v>
+      </c>
+      <c r="C6" s="29" t="s">
+        <v>115</v>
+      </c>
+      <c r="D6" s="29" t="s">
+        <v>116</v>
+      </c>
+      <c r="E6" s="30" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5">
+      <c r="B7" s="29" t="s">
+        <v>117</v>
+      </c>
+      <c r="C7" s="29" t="s">
+        <v>118</v>
+      </c>
+      <c r="D7" s="29" t="s">
+        <v>116</v>
+      </c>
+      <c r="E7" s="29" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5">
+      <c r="B8" s="29" t="s">
+        <v>120</v>
+      </c>
+      <c r="C8" s="29" t="s">
+        <v>121</v>
+      </c>
+      <c r="D8" s="29" t="s">
+        <v>105</v>
+      </c>
+      <c r="E8" s="29" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5">
+      <c r="B9" s="29" t="s">
+        <v>123</v>
+      </c>
+      <c r="C9" s="29" t="s">
+        <v>124</v>
+      </c>
+      <c r="D9" s="29" t="s">
+        <v>105</v>
+      </c>
+      <c r="E9" s="29" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5">
+      <c r="B10" s="29" t="s">
+        <v>126</v>
+      </c>
+      <c r="C10" s="29" t="s">
+        <v>127</v>
+      </c>
+      <c r="D10" s="29" t="s">
+        <v>105</v>
+      </c>
+      <c r="E10" s="29" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5">
+      <c r="B11" s="29" t="s">
+        <v>129</v>
+      </c>
+      <c r="C11" s="29" t="s">
+        <v>130</v>
+      </c>
+      <c r="D11" s="29" t="s">
+        <v>105</v>
+      </c>
+      <c r="E11" s="29" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5">
+      <c r="B12" s="29" t="s">
+        <v>132</v>
+      </c>
+      <c r="C12" s="29" t="s">
+        <v>133</v>
+      </c>
+      <c r="D12" s="29" t="s">
+        <v>105</v>
+      </c>
+      <c r="E12" s="29" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5">
+      <c r="B13" s="29" t="s">
+        <v>135</v>
+      </c>
+      <c r="C13" s="29" t="s">
+        <v>136</v>
+      </c>
+      <c r="D13" s="29" t="s">
+        <v>105</v>
+      </c>
+      <c r="E13" s="29" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5">
+      <c r="B14" s="29" t="s">
+        <v>138</v>
+      </c>
+      <c r="C14" s="29" t="s">
+        <v>139</v>
+      </c>
+      <c r="D14" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="E14" s="29" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5">
+      <c r="B15" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="C15" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="D15" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="E15" s="29" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5">
+      <c r="B16" s="29" t="s">
+        <v>145</v>
+      </c>
+      <c r="C16" s="29" t="s">
+        <v>146</v>
+      </c>
+      <c r="D16" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="E16" s="29" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5">
+      <c r="B17" s="29" t="s">
+        <v>148</v>
+      </c>
+      <c r="C17" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="D17" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="E17" s="29" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5">
+      <c r="B18" s="29" t="s">
+        <v>151</v>
+      </c>
+      <c r="C18" s="29" t="s">
+        <v>152</v>
+      </c>
+      <c r="D18" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="E18" s="29" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5">
+      <c r="B19" s="29" t="s">
+        <v>154</v>
+      </c>
+      <c r="C19" s="29" t="s">
+        <v>155</v>
+      </c>
+      <c r="D19" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="E19" s="29" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5">
+      <c r="B20" s="29" t="s">
+        <v>157</v>
+      </c>
+      <c r="C20" s="29" t="s">
+        <v>158</v>
+      </c>
+      <c r="D20" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="E20" s="29" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5">
+      <c r="B21" s="29" t="s">
+        <v>160</v>
+      </c>
+      <c r="C21" s="29" t="s">
+        <v>161</v>
+      </c>
+      <c r="D21" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="E21" s="29" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5">
+      <c r="B22" s="29" t="s">
+        <v>163</v>
+      </c>
+      <c r="C22" s="29" t="s">
+        <v>164</v>
+      </c>
+      <c r="D22" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="E22" s="29" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5">
+      <c r="B23" s="29" t="s">
+        <v>166</v>
+      </c>
+      <c r="C23" s="29" t="s">
+        <v>167</v>
+      </c>
+      <c r="D23" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="E23" s="29" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5">
+      <c r="B24" s="29" t="s">
+        <v>169</v>
+      </c>
+      <c r="C24" s="29" t="s">
+        <v>170</v>
+      </c>
+      <c r="D24" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="E24" s="29" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5">
+      <c r="B25" s="29" t="s">
+        <v>172</v>
+      </c>
+      <c r="C25" s="29" t="s">
+        <v>173</v>
+      </c>
+      <c r="D25" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="E25" s="29" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5">
+      <c r="B26" s="29" t="s">
+        <v>175</v>
+      </c>
+      <c r="C26" s="29" t="s">
+        <v>176</v>
+      </c>
+      <c r="D26" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="E26" s="29" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5">
+      <c r="B27" s="29" t="s">
+        <v>178</v>
+      </c>
+      <c r="C27" s="29" t="s">
+        <v>179</v>
+      </c>
+      <c r="D27" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="E27" s="29" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="28" spans="2:5">
+      <c r="B28" s="29" t="s">
+        <v>181</v>
+      </c>
+      <c r="C28" s="29" t="s">
+        <v>182</v>
+      </c>
+      <c r="D28" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="E28" s="29" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="29" spans="2:5">
+      <c r="B29" s="29" t="s">
+        <v>184</v>
+      </c>
+      <c r="C29" s="29" t="s">
+        <v>185</v>
+      </c>
+      <c r="D29" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="E29" s="29" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5">
+      <c r="B30" s="29" t="s">
+        <v>187</v>
+      </c>
+      <c r="C30" s="29" t="s">
+        <v>188</v>
+      </c>
+      <c r="D30" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="E30" s="29" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="31" spans="2:5">
+      <c r="B31" s="29" t="s">
+        <v>190</v>
+      </c>
+      <c r="C31" s="29" t="s">
+        <v>191</v>
+      </c>
+      <c r="D31" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="E31" s="29" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5">
+      <c r="B32" s="29" t="s">
+        <v>193</v>
+      </c>
+      <c r="C32" s="29" t="s">
+        <v>194</v>
+      </c>
+      <c r="D32" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="E32" s="29" t="s">
+        <v>195</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
cleaning and updating report.qmd
</commit_message>
<xml_diff>
--- a/Project Plan.xlsx
+++ b/Project Plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Semester 2\ETC5521\Project 1\project-part-1-p1-wallaby\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAD0521C-EA03-4FBC-8B23-36689C979B3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69D20DDA-44B7-4270-B3C4-C431DA2B3B10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="2" xr2:uid="{08FA5D9B-BDCD-4B0C-BBC1-0603E7BA2D97}"/>
+    <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="12863" xr2:uid="{08FA5D9B-BDCD-4B0C-BBC1-0603E7BA2D97}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Plan" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="200">
   <si>
     <t>Section</t>
   </si>
@@ -777,9 +777,6 @@
 3. Size–profitability gradient (log assets vs EBIT margin)</t>
   </si>
   <si>
-    <t>How did firm size influence financial resilience during the pandemic period (2020–2022)?</t>
-  </si>
-  <si>
     <t>How did the fundamental relationship between corporate liquidity and profitability evolve and fracture within industries during the pandemic?</t>
   </si>
   <si>
@@ -1102,13 +1099,22 @@
   </si>
   <si>
     <t>Original Name</t>
+  </si>
+  <si>
+    <t>How did profitability change across industries?</t>
+  </si>
+  <si>
+    <t>How did leverage (debt-to-assets) and liquidity (current ratio) evolve during pandemic?</t>
+  </si>
+  <si>
+    <t>How did firm size influence financial resilience during the pandemic period?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1150,13 +1156,6 @@
       <name val="等线"/>
       <family val="3"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1285,7 +1284,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1320,6 +1319,12 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1359,15 +1364,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1698,31 +1694,31 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10">
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="E2" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="22" t="s">
+      <c r="F2" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
-      <c r="J2" s="24"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+      <c r="I2" s="25"/>
+      <c r="J2" s="26"/>
     </row>
     <row r="3" spans="2:10">
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
       <c r="F3" s="2" t="s">
         <v>12</v>
       </c>
@@ -1740,79 +1736,79 @@
       </c>
     </row>
     <row r="4" spans="2:10" s="5" customFormat="1" ht="20.350000000000001" customHeight="1">
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="21" t="s">
         <v>24</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="25" t="s">
-        <v>32</v>
-      </c>
-      <c r="G4" s="26"/>
-      <c r="H4" s="26"/>
-      <c r="I4" s="26"/>
-      <c r="J4" s="27"/>
+      <c r="F4" s="27" t="s">
+        <v>197</v>
+      </c>
+      <c r="G4" s="28"/>
+      <c r="H4" s="28"/>
+      <c r="I4" s="28"/>
+      <c r="J4" s="29"/>
     </row>
     <row r="5" spans="2:10" s="5" customFormat="1" ht="31.15" customHeight="1">
-      <c r="B5" s="16"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="20"/>
+      <c r="B5" s="18"/>
+      <c r="C5" s="18"/>
+      <c r="D5" s="22"/>
       <c r="E5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="25" t="s">
-        <v>30</v>
-      </c>
-      <c r="G5" s="26"/>
-      <c r="H5" s="26"/>
-      <c r="I5" s="26"/>
-      <c r="J5" s="27"/>
+      <c r="F5" s="27" t="s">
+        <v>198</v>
+      </c>
+      <c r="G5" s="28"/>
+      <c r="H5" s="28"/>
+      <c r="I5" s="28"/>
+      <c r="J5" s="29"/>
     </row>
     <row r="6" spans="2:10" s="5" customFormat="1" ht="30.75" customHeight="1">
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="20"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="22"/>
       <c r="E6" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="25" t="s">
+      <c r="F6" s="27" t="s">
+        <v>199</v>
+      </c>
+      <c r="G6" s="28"/>
+      <c r="H6" s="28"/>
+      <c r="I6" s="28"/>
+      <c r="J6" s="29"/>
+    </row>
+    <row r="7" spans="2:10" s="5" customFormat="1" ht="31.9" customHeight="1">
+      <c r="B7" s="18"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="F7" s="27" t="s">
         <v>94</v>
       </c>
-      <c r="G6" s="26"/>
-      <c r="H6" s="26"/>
-      <c r="I6" s="26"/>
-      <c r="J6" s="27"/>
-    </row>
-    <row r="7" spans="2:10" s="5" customFormat="1" ht="31.9" customHeight="1">
-      <c r="B7" s="16"/>
-      <c r="C7" s="16"/>
-      <c r="D7" s="21"/>
-      <c r="E7" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="F7" s="25" t="s">
-        <v>95</v>
-      </c>
-      <c r="G7" s="26"/>
-      <c r="H7" s="26"/>
-      <c r="I7" s="26"/>
-      <c r="J7" s="27"/>
+      <c r="G7" s="28"/>
+      <c r="H7" s="28"/>
+      <c r="I7" s="28"/>
+      <c r="J7" s="29"/>
     </row>
     <row r="8" spans="2:10">
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="21" t="s">
         <v>25</v>
       </c>
       <c r="E8" s="1" t="s">
@@ -1825,9 +1821,9 @@
       <c r="J8" s="1"/>
     </row>
     <row r="9" spans="2:10">
-      <c r="B9" s="15"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="20"/>
+      <c r="B9" s="17"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="22"/>
       <c r="E9" s="1" t="s">
         <v>9</v>
       </c>
@@ -1838,9 +1834,9 @@
       <c r="J9" s="1"/>
     </row>
     <row r="10" spans="2:10" ht="13.9" customHeight="1">
-      <c r="B10" s="15"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="20"/>
+      <c r="B10" s="17"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="22"/>
       <c r="E10" s="1" t="s">
         <v>10</v>
       </c>
@@ -1851,9 +1847,9 @@
       <c r="J10" s="1"/>
     </row>
     <row r="11" spans="2:10" ht="25.5" customHeight="1">
-      <c r="B11" s="15"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="21"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="23"/>
       <c r="E11" s="1" t="s">
         <v>11</v>
       </c>
@@ -1864,13 +1860,13 @@
       <c r="J11" s="1"/>
     </row>
     <row r="12" spans="2:10">
-      <c r="B12" s="15" t="s">
+      <c r="B12" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="19" t="s">
+      <c r="D12" s="21" t="s">
         <v>26</v>
       </c>
       <c r="E12" s="1" t="s">
@@ -1883,9 +1879,9 @@
       <c r="J12" s="1"/>
     </row>
     <row r="13" spans="2:10">
-      <c r="B13" s="15"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="20"/>
+      <c r="B13" s="17"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="22"/>
       <c r="E13" s="1" t="s">
         <v>9</v>
       </c>
@@ -1896,9 +1892,9 @@
       <c r="J13" s="1"/>
     </row>
     <row r="14" spans="2:10">
-      <c r="B14" s="15"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="20"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="22"/>
       <c r="E14" s="1" t="s">
         <v>10</v>
       </c>
@@ -1909,9 +1905,9 @@
       <c r="J14" s="1"/>
     </row>
     <row r="15" spans="2:10">
-      <c r="B15" s="15"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="21"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="23"/>
       <c r="E15" s="1" t="s">
         <v>11</v>
       </c>
@@ -1922,13 +1918,13 @@
       <c r="J15" s="1"/>
     </row>
     <row r="16" spans="2:10">
-      <c r="B16" s="15" t="s">
+      <c r="B16" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="16" t="s">
+      <c r="C16" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="D16" s="19" t="s">
+      <c r="D16" s="21" t="s">
         <v>27</v>
       </c>
       <c r="E16" s="1" t="s">
@@ -1941,9 +1937,9 @@
       <c r="J16" s="1"/>
     </row>
     <row r="17" spans="2:10">
-      <c r="B17" s="15"/>
-      <c r="C17" s="16"/>
-      <c r="D17" s="20"/>
+      <c r="B17" s="17"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="22"/>
       <c r="E17" s="1" t="s">
         <v>9</v>
       </c>
@@ -1954,9 +1950,9 @@
       <c r="J17" s="1"/>
     </row>
     <row r="18" spans="2:10">
-      <c r="B18" s="15"/>
-      <c r="C18" s="16"/>
-      <c r="D18" s="20"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="22"/>
       <c r="E18" s="1" t="s">
         <v>10</v>
       </c>
@@ -1967,9 +1963,9 @@
       <c r="J18" s="1"/>
     </row>
     <row r="19" spans="2:10" ht="25.15" customHeight="1">
-      <c r="B19" s="15"/>
-      <c r="C19" s="16"/>
-      <c r="D19" s="21"/>
+      <c r="B19" s="17"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="23"/>
       <c r="E19" s="1" t="s">
         <v>11</v>
       </c>
@@ -1980,13 +1976,13 @@
       <c r="J19" s="1"/>
     </row>
     <row r="20" spans="2:10">
-      <c r="B20" s="15" t="s">
+      <c r="B20" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="C20" s="16" t="s">
+      <c r="C20" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="D20" s="19" t="s">
+      <c r="D20" s="21" t="s">
         <v>28</v>
       </c>
       <c r="E20" s="1" t="s">
@@ -1999,9 +1995,9 @@
       <c r="J20" s="1"/>
     </row>
     <row r="21" spans="2:10">
-      <c r="B21" s="15"/>
-      <c r="C21" s="16"/>
-      <c r="D21" s="20"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="22"/>
       <c r="E21" s="1" t="s">
         <v>9</v>
       </c>
@@ -2012,9 +2008,9 @@
       <c r="J21" s="1"/>
     </row>
     <row r="22" spans="2:10">
-      <c r="B22" s="15"/>
-      <c r="C22" s="16"/>
-      <c r="D22" s="20"/>
+      <c r="B22" s="17"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="22"/>
       <c r="E22" s="1" t="s">
         <v>10</v>
       </c>
@@ -2025,9 +2021,9 @@
       <c r="J22" s="1"/>
     </row>
     <row r="23" spans="2:10">
-      <c r="B23" s="15"/>
-      <c r="C23" s="16"/>
-      <c r="D23" s="21"/>
+      <c r="B23" s="17"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="23"/>
       <c r="E23" s="1" t="s">
         <v>11</v>
       </c>
@@ -2097,11 +2093,11 @@
         <v>21</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="2:8" ht="85.5">
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="21" t="s">
         <v>29</v>
       </c>
       <c r="C3" s="4" t="s">
@@ -2120,7 +2116,7 @@
       </c>
     </row>
     <row r="4" spans="2:8" ht="85.5">
-      <c r="B4" s="20"/>
+      <c r="B4" s="22"/>
       <c r="C4" s="4" t="s">
         <v>30</v>
       </c>
@@ -2137,7 +2133,7 @@
       </c>
     </row>
     <row r="5" spans="2:8" ht="85.5">
-      <c r="B5" s="20"/>
+      <c r="B5" s="22"/>
       <c r="C5" s="11" t="s">
         <v>31</v>
       </c>
@@ -2156,14 +2152,14 @@
     <row r="6" spans="2:8" ht="85.5">
       <c r="B6" s="4"/>
       <c r="C6" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E6" s="12"/>
       <c r="F6" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G6" s="12"/>
       <c r="H6" s="12" t="s">
@@ -2544,437 +2540,437 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:5">
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="C2" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="C2" s="28" t="s">
+      <c r="D2" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="D2" s="28" t="s">
+      <c r="E2" s="15" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5">
+      <c r="B3" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="E2" s="28" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="3" spans="2:5">
-      <c r="B3" s="29" t="s">
+      <c r="C3" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="29" t="s">
+      <c r="D3" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="D3" s="29" t="s">
+      <c r="E3" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="E3" s="29" t="s">
+    </row>
+    <row r="4" spans="2:5">
+      <c r="B4" s="4" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="4" spans="2:5">
-      <c r="B4" s="29" t="s">
+      <c r="C4" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="C4" s="29" t="s">
+      <c r="D4" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="E4" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="D4" s="29" t="s">
-        <v>105</v>
-      </c>
-      <c r="E4" s="29" t="s">
+    </row>
+    <row r="5" spans="2:5">
+      <c r="B5" s="4" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="5" spans="2:5">
-      <c r="B5" s="29" t="s">
+      <c r="C5" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="C5" s="29" t="s">
+      <c r="D5" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="E5" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="E5" s="29" t="s">
+    </row>
+    <row r="6" spans="2:5">
+      <c r="B6" s="4" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="6" spans="2:5">
-      <c r="B6" s="29" t="s">
+      <c r="C6" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="D6" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="D6" s="29" t="s">
+      <c r="E6" s="16" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5">
+      <c r="B7" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="E6" s="30" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="7" spans="2:5">
-      <c r="B7" s="29" t="s">
+      <c r="C7" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="C7" s="29" t="s">
+      <c r="D7" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="D7" s="29" t="s">
-        <v>116</v>
-      </c>
-      <c r="E7" s="29" t="s">
+    </row>
+    <row r="8" spans="2:5">
+      <c r="B8" s="4" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="8" spans="2:5">
-      <c r="B8" s="29" t="s">
+      <c r="C8" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="C8" s="29" t="s">
+      <c r="D8" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="E8" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="D8" s="29" t="s">
-        <v>105</v>
-      </c>
-      <c r="E8" s="29" t="s">
+    </row>
+    <row r="9" spans="2:5">
+      <c r="B9" s="4" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="9" spans="2:5">
-      <c r="B9" s="29" t="s">
+      <c r="C9" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="C9" s="29" t="s">
+      <c r="D9" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="E9" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="D9" s="29" t="s">
-        <v>105</v>
-      </c>
-      <c r="E9" s="29" t="s">
+    </row>
+    <row r="10" spans="2:5">
+      <c r="B10" s="4" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="10" spans="2:5">
-      <c r="B10" s="29" t="s">
+      <c r="C10" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="C10" s="29" t="s">
+      <c r="D10" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="E10" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="D10" s="29" t="s">
-        <v>105</v>
-      </c>
-      <c r="E10" s="29" t="s">
+    </row>
+    <row r="11" spans="2:5">
+      <c r="B11" s="4" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="11" spans="2:5">
-      <c r="B11" s="29" t="s">
+      <c r="C11" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="C11" s="29" t="s">
+      <c r="D11" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="E11" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="D11" s="29" t="s">
-        <v>105</v>
-      </c>
-      <c r="E11" s="29" t="s">
+    </row>
+    <row r="12" spans="2:5">
+      <c r="B12" s="4" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="12" spans="2:5">
-      <c r="B12" s="29" t="s">
+      <c r="C12" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="C12" s="29" t="s">
+      <c r="D12" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="E12" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="D12" s="29" t="s">
-        <v>105</v>
-      </c>
-      <c r="E12" s="29" t="s">
+    </row>
+    <row r="13" spans="2:5">
+      <c r="B13" s="4" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="13" spans="2:5">
-      <c r="B13" s="29" t="s">
+      <c r="C13" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="C13" s="29" t="s">
+      <c r="D13" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="E13" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="D13" s="29" t="s">
-        <v>105</v>
-      </c>
-      <c r="E13" s="29" t="s">
+    </row>
+    <row r="14" spans="2:5">
+      <c r="B14" s="4" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="14" spans="2:5">
-      <c r="B14" s="29" t="s">
+      <c r="C14" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="C14" s="29" t="s">
+      <c r="D14" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="D14" s="29" t="s">
+      <c r="E14" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="E14" s="29" t="s">
+    </row>
+    <row r="15" spans="2:5">
+      <c r="B15" s="4" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="15" spans="2:5">
-      <c r="B15" s="29" t="s">
+      <c r="C15" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="C15" s="29" t="s">
+      <c r="D15" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E15" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="D15" s="29" t="s">
-        <v>140</v>
-      </c>
-      <c r="E15" s="29" t="s">
+    </row>
+    <row r="16" spans="2:5">
+      <c r="B16" s="4" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="16" spans="2:5">
-      <c r="B16" s="29" t="s">
+      <c r="C16" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="C16" s="29" t="s">
+      <c r="D16" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E16" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="D16" s="29" t="s">
-        <v>140</v>
-      </c>
-      <c r="E16" s="29" t="s">
+    </row>
+    <row r="17" spans="2:5">
+      <c r="B17" s="4" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="17" spans="2:5">
-      <c r="B17" s="29" t="s">
+      <c r="C17" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="C17" s="29" t="s">
+      <c r="D17" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E17" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="D17" s="29" t="s">
-        <v>140</v>
-      </c>
-      <c r="E17" s="29" t="s">
+    </row>
+    <row r="18" spans="2:5">
+      <c r="B18" s="4" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="18" spans="2:5">
-      <c r="B18" s="29" t="s">
+      <c r="C18" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="C18" s="29" t="s">
+      <c r="D18" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E18" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="D18" s="29" t="s">
-        <v>140</v>
-      </c>
-      <c r="E18" s="29" t="s">
+    </row>
+    <row r="19" spans="2:5">
+      <c r="B19" s="4" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="19" spans="2:5">
-      <c r="B19" s="29" t="s">
+      <c r="C19" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="C19" s="29" t="s">
+      <c r="D19" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E19" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="D19" s="29" t="s">
-        <v>140</v>
-      </c>
-      <c r="E19" s="29" t="s">
+    </row>
+    <row r="20" spans="2:5">
+      <c r="B20" s="4" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="20" spans="2:5">
-      <c r="B20" s="29" t="s">
+      <c r="C20" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="C20" s="29" t="s">
+      <c r="D20" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E20" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="D20" s="29" t="s">
-        <v>140</v>
-      </c>
-      <c r="E20" s="29" t="s">
+    </row>
+    <row r="21" spans="2:5">
+      <c r="B21" s="4" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="21" spans="2:5">
-      <c r="B21" s="29" t="s">
+      <c r="C21" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="C21" s="29" t="s">
+      <c r="D21" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E21" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="D21" s="29" t="s">
-        <v>140</v>
-      </c>
-      <c r="E21" s="29" t="s">
+    </row>
+    <row r="22" spans="2:5">
+      <c r="B22" s="4" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="22" spans="2:5">
-      <c r="B22" s="29" t="s">
+      <c r="C22" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="C22" s="29" t="s">
+      <c r="D22" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E22" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="D22" s="29" t="s">
-        <v>140</v>
-      </c>
-      <c r="E22" s="29" t="s">
+    </row>
+    <row r="23" spans="2:5">
+      <c r="B23" s="4" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="23" spans="2:5">
-      <c r="B23" s="29" t="s">
+      <c r="C23" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="C23" s="29" t="s">
+      <c r="D23" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E23" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="D23" s="29" t="s">
-        <v>140</v>
-      </c>
-      <c r="E23" s="29" t="s">
+    </row>
+    <row r="24" spans="2:5">
+      <c r="B24" s="4" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="24" spans="2:5">
-      <c r="B24" s="29" t="s">
+      <c r="C24" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="C24" s="29" t="s">
+      <c r="D24" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E24" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="D24" s="29" t="s">
-        <v>140</v>
-      </c>
-      <c r="E24" s="29" t="s">
+    </row>
+    <row r="25" spans="2:5">
+      <c r="B25" s="4" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="25" spans="2:5">
-      <c r="B25" s="29" t="s">
+      <c r="C25" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="C25" s="29" t="s">
+      <c r="D25" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E25" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="D25" s="29" t="s">
-        <v>140</v>
-      </c>
-      <c r="E25" s="29" t="s">
+    </row>
+    <row r="26" spans="2:5">
+      <c r="B26" s="4" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="26" spans="2:5">
-      <c r="B26" s="29" t="s">
+      <c r="C26" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="C26" s="29" t="s">
+      <c r="D26" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E26" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="D26" s="29" t="s">
-        <v>140</v>
-      </c>
-      <c r="E26" s="29" t="s">
+    </row>
+    <row r="27" spans="2:5">
+      <c r="B27" s="4" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="27" spans="2:5">
-      <c r="B27" s="29" t="s">
+      <c r="C27" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="C27" s="29" t="s">
+      <c r="D27" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E27" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="D27" s="29" t="s">
-        <v>140</v>
-      </c>
-      <c r="E27" s="29" t="s">
+    </row>
+    <row r="28" spans="2:5">
+      <c r="B28" s="4" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="28" spans="2:5">
-      <c r="B28" s="29" t="s">
+      <c r="C28" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C28" s="29" t="s">
+      <c r="D28" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E28" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="D28" s="29" t="s">
-        <v>140</v>
-      </c>
-      <c r="E28" s="29" t="s">
+    </row>
+    <row r="29" spans="2:5">
+      <c r="B29" s="4" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="29" spans="2:5">
-      <c r="B29" s="29" t="s">
+      <c r="C29" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="C29" s="29" t="s">
+      <c r="D29" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E29" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="D29" s="29" t="s">
-        <v>140</v>
-      </c>
-      <c r="E29" s="29" t="s">
+    </row>
+    <row r="30" spans="2:5">
+      <c r="B30" s="4" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="30" spans="2:5">
-      <c r="B30" s="29" t="s">
+      <c r="C30" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="C30" s="29" t="s">
+      <c r="D30" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E30" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="D30" s="29" t="s">
-        <v>140</v>
-      </c>
-      <c r="E30" s="29" t="s">
+    </row>
+    <row r="31" spans="2:5">
+      <c r="B31" s="4" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="31" spans="2:5">
-      <c r="B31" s="29" t="s">
+      <c r="C31" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="C31" s="29" t="s">
+      <c r="D31" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E31" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="D31" s="29" t="s">
-        <v>140</v>
-      </c>
-      <c r="E31" s="29" t="s">
+    </row>
+    <row r="32" spans="2:5">
+      <c r="B32" s="4" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="32" spans="2:5">
-      <c r="B32" s="29" t="s">
+      <c r="C32" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="C32" s="29" t="s">
+      <c r="D32" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E32" s="4" t="s">
         <v>194</v>
-      </c>
-      <c r="D32" s="29" t="s">
-        <v>140</v>
-      </c>
-      <c r="E32" s="29" t="s">
-        <v>195</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updating EDA results for Question 1 (chart 1 and 2)
</commit_message>
<xml_diff>
--- a/Project Plan.xlsx
+++ b/Project Plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Semester 2\ETC5521\Project 1\project-part-1-p1-wallaby\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69D20DDA-44B7-4270-B3C4-C431DA2B3B10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A249451-398D-4BF1-9746-1B474FB6DC47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="12863" xr2:uid="{08FA5D9B-BDCD-4B0C-BBC1-0603E7BA2D97}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{08FA5D9B-BDCD-4B0C-BBC1-0603E7BA2D97}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Plan" sheetId="1" r:id="rId1"/>
@@ -1326,18 +1326,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1346,6 +1334,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1364,6 +1358,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1694,31 +1694,31 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10">
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="19" t="s">
+      <c r="D2" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="19" t="s">
+      <c r="E2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="24" t="s">
+      <c r="F2" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="26"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="24"/>
     </row>
     <row r="3" spans="2:10">
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
       <c r="F3" s="2" t="s">
         <v>12</v>
       </c>
@@ -1736,79 +1736,79 @@
       </c>
     </row>
     <row r="4" spans="2:10" s="5" customFormat="1" ht="20.350000000000001" customHeight="1">
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="21" t="s">
+      <c r="D4" s="17" t="s">
         <v>24</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="27" t="s">
+      <c r="F4" s="25" t="s">
         <v>197</v>
       </c>
-      <c r="G4" s="28"/>
-      <c r="H4" s="28"/>
-      <c r="I4" s="28"/>
-      <c r="J4" s="29"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="26"/>
+      <c r="I4" s="26"/>
+      <c r="J4" s="27"/>
     </row>
     <row r="5" spans="2:10" s="5" customFormat="1" ht="31.15" customHeight="1">
-      <c r="B5" s="18"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="22"/>
+      <c r="B5" s="29"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="18"/>
       <c r="E5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="27" t="s">
+      <c r="F5" s="25" t="s">
         <v>198</v>
       </c>
-      <c r="G5" s="28"/>
-      <c r="H5" s="28"/>
-      <c r="I5" s="28"/>
-      <c r="J5" s="29"/>
+      <c r="G5" s="26"/>
+      <c r="H5" s="26"/>
+      <c r="I5" s="26"/>
+      <c r="J5" s="27"/>
     </row>
     <row r="6" spans="2:10" s="5" customFormat="1" ht="30.75" customHeight="1">
-      <c r="B6" s="18"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="22"/>
+      <c r="B6" s="29"/>
+      <c r="C6" s="29"/>
+      <c r="D6" s="18"/>
       <c r="E6" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="27" t="s">
+      <c r="F6" s="25" t="s">
         <v>199</v>
       </c>
-      <c r="G6" s="28"/>
-      <c r="H6" s="28"/>
-      <c r="I6" s="28"/>
-      <c r="J6" s="29"/>
+      <c r="G6" s="26"/>
+      <c r="H6" s="26"/>
+      <c r="I6" s="26"/>
+      <c r="J6" s="27"/>
     </row>
     <row r="7" spans="2:10" s="5" customFormat="1" ht="31.9" customHeight="1">
-      <c r="B7" s="18"/>
-      <c r="C7" s="18"/>
-      <c r="D7" s="23"/>
+      <c r="B7" s="29"/>
+      <c r="C7" s="29"/>
+      <c r="D7" s="19"/>
       <c r="E7" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="F7" s="27" t="s">
+      <c r="F7" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="G7" s="28"/>
-      <c r="H7" s="28"/>
-      <c r="I7" s="28"/>
-      <c r="J7" s="29"/>
+      <c r="G7" s="26"/>
+      <c r="H7" s="26"/>
+      <c r="I7" s="26"/>
+      <c r="J7" s="27"/>
     </row>
     <row r="8" spans="2:10">
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="21" t="s">
+      <c r="D8" s="17" t="s">
         <v>25</v>
       </c>
       <c r="E8" s="1" t="s">
@@ -1821,9 +1821,9 @@
       <c r="J8" s="1"/>
     </row>
     <row r="9" spans="2:10">
-      <c r="B9" s="17"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="22"/>
+      <c r="B9" s="28"/>
+      <c r="C9" s="29"/>
+      <c r="D9" s="18"/>
       <c r="E9" s="1" t="s">
         <v>9</v>
       </c>
@@ -1834,9 +1834,9 @@
       <c r="J9" s="1"/>
     </row>
     <row r="10" spans="2:10" ht="13.9" customHeight="1">
-      <c r="B10" s="17"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="22"/>
+      <c r="B10" s="28"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="18"/>
       <c r="E10" s="1" t="s">
         <v>10</v>
       </c>
@@ -1847,9 +1847,9 @@
       <c r="J10" s="1"/>
     </row>
     <row r="11" spans="2:10" ht="25.5" customHeight="1">
-      <c r="B11" s="17"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="23"/>
+      <c r="B11" s="28"/>
+      <c r="C11" s="29"/>
+      <c r="D11" s="19"/>
       <c r="E11" s="1" t="s">
         <v>11</v>
       </c>
@@ -1860,13 +1860,13 @@
       <c r="J11" s="1"/>
     </row>
     <row r="12" spans="2:10">
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="21" t="s">
+      <c r="D12" s="17" t="s">
         <v>26</v>
       </c>
       <c r="E12" s="1" t="s">
@@ -1879,9 +1879,9 @@
       <c r="J12" s="1"/>
     </row>
     <row r="13" spans="2:10">
-      <c r="B13" s="17"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="22"/>
+      <c r="B13" s="28"/>
+      <c r="C13" s="29"/>
+      <c r="D13" s="18"/>
       <c r="E13" s="1" t="s">
         <v>9</v>
       </c>
@@ -1892,9 +1892,9 @@
       <c r="J13" s="1"/>
     </row>
     <row r="14" spans="2:10">
-      <c r="B14" s="17"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="22"/>
+      <c r="B14" s="28"/>
+      <c r="C14" s="29"/>
+      <c r="D14" s="18"/>
       <c r="E14" s="1" t="s">
         <v>10</v>
       </c>
@@ -1905,9 +1905,9 @@
       <c r="J14" s="1"/>
     </row>
     <row r="15" spans="2:10">
-      <c r="B15" s="17"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="23"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="19"/>
       <c r="E15" s="1" t="s">
         <v>11</v>
       </c>
@@ -1918,13 +1918,13 @@
       <c r="J15" s="1"/>
     </row>
     <row r="16" spans="2:10">
-      <c r="B16" s="17" t="s">
+      <c r="B16" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="C16" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="D16" s="21" t="s">
+      <c r="D16" s="17" t="s">
         <v>27</v>
       </c>
       <c r="E16" s="1" t="s">
@@ -1937,9 +1937,9 @@
       <c r="J16" s="1"/>
     </row>
     <row r="17" spans="2:10">
-      <c r="B17" s="17"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="22"/>
+      <c r="B17" s="28"/>
+      <c r="C17" s="29"/>
+      <c r="D17" s="18"/>
       <c r="E17" s="1" t="s">
         <v>9</v>
       </c>
@@ -1950,9 +1950,9 @@
       <c r="J17" s="1"/>
     </row>
     <row r="18" spans="2:10">
-      <c r="B18" s="17"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="22"/>
+      <c r="B18" s="28"/>
+      <c r="C18" s="29"/>
+      <c r="D18" s="18"/>
       <c r="E18" s="1" t="s">
         <v>10</v>
       </c>
@@ -1963,9 +1963,9 @@
       <c r="J18" s="1"/>
     </row>
     <row r="19" spans="2:10" ht="25.15" customHeight="1">
-      <c r="B19" s="17"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="23"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="19"/>
       <c r="E19" s="1" t="s">
         <v>11</v>
       </c>
@@ -1976,13 +1976,13 @@
       <c r="J19" s="1"/>
     </row>
     <row r="20" spans="2:10">
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="C20" s="18" t="s">
+      <c r="C20" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="D20" s="21" t="s">
+      <c r="D20" s="17" t="s">
         <v>28</v>
       </c>
       <c r="E20" s="1" t="s">
@@ -1995,9 +1995,9 @@
       <c r="J20" s="1"/>
     </row>
     <row r="21" spans="2:10">
-      <c r="B21" s="17"/>
-      <c r="C21" s="18"/>
-      <c r="D21" s="22"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="18"/>
       <c r="E21" s="1" t="s">
         <v>9</v>
       </c>
@@ -2008,9 +2008,9 @@
       <c r="J21" s="1"/>
     </row>
     <row r="22" spans="2:10">
-      <c r="B22" s="17"/>
-      <c r="C22" s="18"/>
-      <c r="D22" s="22"/>
+      <c r="B22" s="28"/>
+      <c r="C22" s="29"/>
+      <c r="D22" s="18"/>
       <c r="E22" s="1" t="s">
         <v>10</v>
       </c>
@@ -2021,9 +2021,9 @@
       <c r="J22" s="1"/>
     </row>
     <row r="23" spans="2:10">
-      <c r="B23" s="17"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="23"/>
+      <c r="B23" s="28"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="19"/>
       <c r="E23" s="1" t="s">
         <v>11</v>
       </c>
@@ -2035,6 +2035,18 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="B16:B19"/>
+    <mergeCell ref="C16:C19"/>
+    <mergeCell ref="C20:C23"/>
+    <mergeCell ref="B20:B23"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="B4:B7"/>
+    <mergeCell ref="C4:C7"/>
+    <mergeCell ref="C8:C11"/>
+    <mergeCell ref="C12:C15"/>
+    <mergeCell ref="B8:B11"/>
+    <mergeCell ref="B12:B15"/>
     <mergeCell ref="D16:D19"/>
     <mergeCell ref="D20:D23"/>
     <mergeCell ref="E2:E3"/>
@@ -2047,18 +2059,6 @@
     <mergeCell ref="F5:J5"/>
     <mergeCell ref="F6:J6"/>
     <mergeCell ref="F7:J7"/>
-    <mergeCell ref="B16:B19"/>
-    <mergeCell ref="C16:C19"/>
-    <mergeCell ref="C20:C23"/>
-    <mergeCell ref="B20:B23"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="B4:B7"/>
-    <mergeCell ref="C4:C7"/>
-    <mergeCell ref="C8:C11"/>
-    <mergeCell ref="C12:C15"/>
-    <mergeCell ref="B8:B11"/>
-    <mergeCell ref="B12:B15"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2097,7 +2097,7 @@
       </c>
     </row>
     <row r="3" spans="2:8" ht="85.5">
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="17" t="s">
         <v>29</v>
       </c>
       <c r="C3" s="4" t="s">
@@ -2116,7 +2116,7 @@
       </c>
     </row>
     <row r="4" spans="2:8" ht="85.5">
-      <c r="B4" s="22"/>
+      <c r="B4" s="18"/>
       <c r="C4" s="4" t="s">
         <v>30</v>
       </c>
@@ -2133,7 +2133,7 @@
       </c>
     </row>
     <row r="5" spans="2:8" ht="85.5">
-      <c r="B5" s="22"/>
+      <c r="B5" s="18"/>
       <c r="C5" s="11" t="s">
         <v>31</v>
       </c>

</xml_diff>